<commit_message>
Deploy: Актуализация форм 42b442323863f89db2f69c5fb418f649e6acd2eb
</commit_message>
<xml_diff>
--- a/docs/forms/форма-10.1.xlsx
+++ b/docs/forms/форма-10.1.xlsx
@@ -1,11 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{098FD2B6-D6F2-432B-B04B-DD5B4F167F04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="p4dwbcdDObro2P8Wzf1VSjM8GirUn1PRozxgtaZFXBduF4jNcaceDSXZy45Ggjuyx9zI6IpcdvibyCPsUj+2EA==" workbookSaltValue="KgM4gtQFlLVKgjUw5SJHsA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Форма № 10.1 прокладка КЛ" sheetId="6" r:id="rId1"/>
@@ -14,11 +15,16 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Форма № 10.1 прокладка КЛ'!$A$1:$AI$66</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="122">
   <si>
     <t>Ф.И.О. указывать полностью</t>
   </si>
@@ -453,7 +459,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="31" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1112,7 +1118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="201">
+  <cellXfs count="204">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1360,11 +1366,44 @@
     <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="17" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
@@ -1374,11 +1413,26 @@
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="17" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
@@ -1396,125 +1450,74 @@
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
@@ -1562,6 +1565,12 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1605,116 +1614,124 @@
     <xf numFmtId="0" fontId="30" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1750,7 +1767,13 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="Овал 1"/>
+        <xdr:cNvPr id="2" name="Овал 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -1876,6 +1899,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -1911,6 +1951,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Стандартная">
@@ -2086,7 +2143,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AS73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2105,119 +2162,119 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="187" t="s">
+      <c r="A1" s="96" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="187"/>
-      <c r="C1" s="187"/>
-      <c r="D1" s="187"/>
-      <c r="E1" s="187"/>
-      <c r="F1" s="187"/>
-      <c r="G1" s="187"/>
-      <c r="H1" s="187"/>
-      <c r="I1" s="187"/>
-      <c r="J1" s="187"/>
-      <c r="K1" s="187"/>
-      <c r="L1" s="187"/>
-      <c r="M1" s="187"/>
-      <c r="N1" s="187"/>
-      <c r="O1" s="187"/>
-      <c r="P1" s="187"/>
-      <c r="Q1" s="187"/>
-      <c r="R1" s="187"/>
-      <c r="S1" s="187"/>
-      <c r="T1" s="187"/>
-      <c r="U1" s="187"/>
-      <c r="V1" s="187"/>
-      <c r="W1" s="187"/>
-      <c r="X1" s="187"/>
-      <c r="Y1" s="187"/>
-      <c r="Z1" s="187"/>
-      <c r="AA1" s="187"/>
-      <c r="AB1" s="187"/>
-      <c r="AC1" s="187"/>
-      <c r="AD1" s="187"/>
-      <c r="AE1" s="187"/>
-      <c r="AF1" s="187"/>
-      <c r="AG1" s="187"/>
-      <c r="AH1" s="187"/>
-      <c r="AI1" s="187"/>
+      <c r="B1" s="96"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="96"/>
+      <c r="G1" s="96"/>
+      <c r="H1" s="96"/>
+      <c r="I1" s="96"/>
+      <c r="J1" s="96"/>
+      <c r="K1" s="96"/>
+      <c r="L1" s="96"/>
+      <c r="M1" s="96"/>
+      <c r="N1" s="96"/>
+      <c r="O1" s="96"/>
+      <c r="P1" s="96"/>
+      <c r="Q1" s="96"/>
+      <c r="R1" s="96"/>
+      <c r="S1" s="96"/>
+      <c r="T1" s="96"/>
+      <c r="U1" s="96"/>
+      <c r="V1" s="96"/>
+      <c r="W1" s="96"/>
+      <c r="X1" s="96"/>
+      <c r="Y1" s="96"/>
+      <c r="Z1" s="96"/>
+      <c r="AA1" s="96"/>
+      <c r="AB1" s="96"/>
+      <c r="AC1" s="96"/>
+      <c r="AD1" s="96"/>
+      <c r="AE1" s="96"/>
+      <c r="AF1" s="96"/>
+      <c r="AG1" s="96"/>
+      <c r="AH1" s="96"/>
+      <c r="AI1" s="96"/>
     </row>
     <row r="2" spans="1:45" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="188" t="s">
+      <c r="A2" s="97" t="s">
         <v>119</v>
       </c>
-      <c r="B2" s="188"/>
-      <c r="C2" s="188"/>
-      <c r="D2" s="188"/>
-      <c r="E2" s="188"/>
-      <c r="F2" s="188"/>
-      <c r="G2" s="188"/>
-      <c r="H2" s="188"/>
-      <c r="I2" s="188"/>
-      <c r="J2" s="188"/>
-      <c r="K2" s="188"/>
-      <c r="L2" s="188"/>
-      <c r="M2" s="188"/>
-      <c r="N2" s="188"/>
-      <c r="O2" s="188"/>
-      <c r="P2" s="188"/>
-      <c r="Q2" s="188"/>
-      <c r="R2" s="188"/>
-      <c r="S2" s="188"/>
-      <c r="T2" s="188"/>
-      <c r="U2" s="188"/>
-      <c r="V2" s="188"/>
-      <c r="W2" s="188"/>
-      <c r="X2" s="188"/>
-      <c r="Y2" s="188"/>
-      <c r="Z2" s="188"/>
-      <c r="AA2" s="188"/>
-      <c r="AB2" s="188"/>
-      <c r="AC2" s="188"/>
-      <c r="AD2" s="188"/>
-      <c r="AE2" s="188"/>
-      <c r="AF2" s="188"/>
-      <c r="AG2" s="188"/>
-      <c r="AH2" s="188"/>
-      <c r="AI2" s="188"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
+      <c r="J2" s="97"/>
+      <c r="K2" s="97"/>
+      <c r="L2" s="97"/>
+      <c r="M2" s="97"/>
+      <c r="N2" s="97"/>
+      <c r="O2" s="97"/>
+      <c r="P2" s="97"/>
+      <c r="Q2" s="97"/>
+      <c r="R2" s="97"/>
+      <c r="S2" s="97"/>
+      <c r="T2" s="97"/>
+      <c r="U2" s="97"/>
+      <c r="V2" s="97"/>
+      <c r="W2" s="97"/>
+      <c r="X2" s="97"/>
+      <c r="Y2" s="97"/>
+      <c r="Z2" s="97"/>
+      <c r="AA2" s="97"/>
+      <c r="AB2" s="97"/>
+      <c r="AC2" s="97"/>
+      <c r="AD2" s="97"/>
+      <c r="AE2" s="97"/>
+      <c r="AF2" s="97"/>
+      <c r="AG2" s="97"/>
+      <c r="AH2" s="97"/>
+      <c r="AI2" s="97"/>
     </row>
     <row r="3" spans="1:45" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="189"/>
-      <c r="B3" s="189"/>
-      <c r="C3" s="189"/>
-      <c r="D3" s="189"/>
-      <c r="E3" s="189"/>
-      <c r="F3" s="189"/>
-      <c r="G3" s="189"/>
-      <c r="H3" s="189"/>
-      <c r="I3" s="189"/>
-      <c r="J3" s="189"/>
-      <c r="K3" s="189"/>
-      <c r="L3" s="189"/>
-      <c r="M3" s="189"/>
-      <c r="N3" s="189"/>
-      <c r="O3" s="189"/>
-      <c r="P3" s="189"/>
-      <c r="Q3" s="189"/>
-      <c r="R3" s="189"/>
-      <c r="S3" s="189"/>
-      <c r="T3" s="189"/>
-      <c r="U3" s="189"/>
-      <c r="V3" s="189"/>
-      <c r="W3" s="189"/>
-      <c r="X3" s="189"/>
-      <c r="Y3" s="189"/>
-      <c r="Z3" s="189"/>
-      <c r="AA3" s="189"/>
-      <c r="AB3" s="189"/>
-      <c r="AC3" s="189"/>
-      <c r="AD3" s="189"/>
-      <c r="AE3" s="189"/>
-      <c r="AF3" s="189"/>
-      <c r="AG3" s="189"/>
-      <c r="AH3" s="189"/>
-      <c r="AI3" s="189"/>
+      <c r="A3" s="98"/>
+      <c r="B3" s="98"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="98"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="98"/>
+      <c r="I3" s="98"/>
+      <c r="J3" s="98"/>
+      <c r="K3" s="98"/>
+      <c r="L3" s="98"/>
+      <c r="M3" s="98"/>
+      <c r="N3" s="98"/>
+      <c r="O3" s="98"/>
+      <c r="P3" s="98"/>
+      <c r="Q3" s="98"/>
+      <c r="R3" s="98"/>
+      <c r="S3" s="98"/>
+      <c r="T3" s="98"/>
+      <c r="U3" s="98"/>
+      <c r="V3" s="98"/>
+      <c r="W3" s="98"/>
+      <c r="X3" s="98"/>
+      <c r="Y3" s="98"/>
+      <c r="Z3" s="98"/>
+      <c r="AA3" s="98"/>
+      <c r="AB3" s="98"/>
+      <c r="AC3" s="98"/>
+      <c r="AD3" s="98"/>
+      <c r="AE3" s="98"/>
+      <c r="AF3" s="98"/>
+      <c r="AG3" s="98"/>
+      <c r="AH3" s="98"/>
+      <c r="AI3" s="98"/>
     </row>
     <row r="4" spans="1:45" s="2" customFormat="1" ht="4.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6"/>
@@ -2270,33 +2327,33 @@
       <c r="A5" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="190" t="s">
+      <c r="B5" s="99" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="190"/>
-      <c r="D5" s="190"/>
-      <c r="E5" s="190"/>
-      <c r="F5" s="190"/>
-      <c r="G5" s="190"/>
-      <c r="H5" s="190"/>
-      <c r="I5" s="190"/>
-      <c r="J5" s="191"/>
-      <c r="K5" s="192"/>
-      <c r="L5" s="192"/>
-      <c r="M5" s="192"/>
-      <c r="N5" s="192"/>
-      <c r="O5" s="192"/>
-      <c r="P5" s="192"/>
-      <c r="Q5" s="192"/>
-      <c r="R5" s="192"/>
-      <c r="S5" s="192"/>
-      <c r="T5" s="192"/>
-      <c r="U5" s="192"/>
-      <c r="V5" s="193"/>
-      <c r="W5" s="194" t="s">
+      <c r="C5" s="99"/>
+      <c r="D5" s="99"/>
+      <c r="E5" s="99"/>
+      <c r="F5" s="99"/>
+      <c r="G5" s="99"/>
+      <c r="H5" s="99"/>
+      <c r="I5" s="99"/>
+      <c r="J5" s="100"/>
+      <c r="K5" s="101"/>
+      <c r="L5" s="101"/>
+      <c r="M5" s="101"/>
+      <c r="N5" s="101"/>
+      <c r="O5" s="101"/>
+      <c r="P5" s="101"/>
+      <c r="Q5" s="101"/>
+      <c r="R5" s="101"/>
+      <c r="S5" s="101"/>
+      <c r="T5" s="101"/>
+      <c r="U5" s="101"/>
+      <c r="V5" s="102"/>
+      <c r="W5" s="103" t="s">
         <v>12</v>
       </c>
-      <c r="X5" s="194"/>
+      <c r="X5" s="103"/>
       <c r="Y5" s="66"/>
       <c r="Z5" s="66"/>
       <c r="AA5" s="66"/>
@@ -2345,21 +2402,21 @@
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
-      <c r="J6" s="195" t="s">
+      <c r="J6" s="104" t="s">
         <v>28</v>
       </c>
-      <c r="K6" s="195"/>
-      <c r="L6" s="195"/>
-      <c r="M6" s="195"/>
-      <c r="N6" s="195"/>
-      <c r="O6" s="195"/>
-      <c r="P6" s="195"/>
-      <c r="Q6" s="195"/>
-      <c r="R6" s="195"/>
-      <c r="S6" s="195"/>
-      <c r="T6" s="195"/>
-      <c r="U6" s="195"/>
-      <c r="V6" s="195"/>
+      <c r="K6" s="104"/>
+      <c r="L6" s="104"/>
+      <c r="M6" s="104"/>
+      <c r="N6" s="104"/>
+      <c r="O6" s="104"/>
+      <c r="P6" s="104"/>
+      <c r="Q6" s="104"/>
+      <c r="R6" s="104"/>
+      <c r="S6" s="104"/>
+      <c r="T6" s="104"/>
+      <c r="U6" s="104"/>
+      <c r="V6" s="104"/>
       <c r="W6" s="10"/>
       <c r="X6" s="10"/>
       <c r="Y6" s="10"/>
@@ -2402,10 +2459,10 @@
     </row>
     <row r="7" spans="1:45" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
-      <c r="B7" s="185" t="s">
+      <c r="B7" s="94" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="185"/>
+      <c r="C7" s="94"/>
       <c r="D7" s="67"/>
       <c r="E7" s="67"/>
       <c r="F7" s="66"/>
@@ -2419,10 +2476,10 @@
       <c r="N7" s="67"/>
       <c r="O7" s="67"/>
       <c r="P7" s="67"/>
-      <c r="Q7" s="186" t="s">
+      <c r="Q7" s="95" t="s">
         <v>13</v>
       </c>
-      <c r="R7" s="186"/>
+      <c r="R7" s="95"/>
       <c r="S7" s="67"/>
       <c r="T7" s="67"/>
       <c r="U7" s="67"/>
@@ -2532,41 +2589,41 @@
     </row>
     <row r="9" spans="1:45" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
-      <c r="B9" s="200" t="s">
+      <c r="B9" s="113" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="200"/>
-      <c r="D9" s="200"/>
-      <c r="E9" s="200"/>
-      <c r="F9" s="200"/>
-      <c r="G9" s="200"/>
-      <c r="H9" s="200"/>
-      <c r="I9" s="100"/>
-      <c r="J9" s="101"/>
-      <c r="K9" s="101"/>
-      <c r="L9" s="101"/>
-      <c r="M9" s="102"/>
+      <c r="C9" s="113"/>
+      <c r="D9" s="113"/>
+      <c r="E9" s="113"/>
+      <c r="F9" s="113"/>
+      <c r="G9" s="113"/>
+      <c r="H9" s="113"/>
+      <c r="I9" s="114"/>
+      <c r="J9" s="115"/>
+      <c r="K9" s="115"/>
+      <c r="L9" s="115"/>
+      <c r="M9" s="116"/>
       <c r="N9" s="72"/>
-      <c r="O9" s="96"/>
-      <c r="P9" s="103"/>
-      <c r="Q9" s="103"/>
-      <c r="R9" s="103"/>
-      <c r="S9" s="103"/>
-      <c r="T9" s="103"/>
-      <c r="U9" s="103"/>
-      <c r="V9" s="103"/>
-      <c r="W9" s="103"/>
-      <c r="X9" s="103"/>
-      <c r="Y9" s="97"/>
+      <c r="O9" s="106"/>
+      <c r="P9" s="117"/>
+      <c r="Q9" s="117"/>
+      <c r="R9" s="117"/>
+      <c r="S9" s="117"/>
+      <c r="T9" s="117"/>
+      <c r="U9" s="117"/>
+      <c r="V9" s="117"/>
+      <c r="W9" s="117"/>
+      <c r="X9" s="117"/>
+      <c r="Y9" s="107"/>
       <c r="Z9" s="72"/>
-      <c r="AA9" s="96"/>
-      <c r="AB9" s="97"/>
+      <c r="AA9" s="106"/>
+      <c r="AB9" s="107"/>
       <c r="AC9" s="73"/>
-      <c r="AD9" s="96"/>
-      <c r="AE9" s="97"/>
+      <c r="AD9" s="106"/>
+      <c r="AE9" s="107"/>
       <c r="AF9" s="72"/>
-      <c r="AG9" s="96"/>
-      <c r="AH9" s="97"/>
+      <c r="AG9" s="106"/>
+      <c r="AH9" s="107"/>
       <c r="AI9" s="9"/>
       <c r="AJ9" s="85"/>
       <c r="AK9" s="85"/>
@@ -2600,42 +2657,42 @@
       <c r="F10" s="15"/>
       <c r="G10" s="15"/>
       <c r="H10" s="15"/>
-      <c r="I10" s="181" t="s">
+      <c r="I10" s="119" t="s">
         <v>48</v>
       </c>
-      <c r="J10" s="181"/>
-      <c r="K10" s="181"/>
-      <c r="L10" s="181"/>
-      <c r="M10" s="181"/>
+      <c r="J10" s="119"/>
+      <c r="K10" s="119"/>
+      <c r="L10" s="119"/>
+      <c r="M10" s="119"/>
       <c r="N10" s="15"/>
-      <c r="O10" s="182" t="s">
+      <c r="O10" s="120" t="s">
         <v>49</v>
       </c>
-      <c r="P10" s="181"/>
-      <c r="Q10" s="181"/>
-      <c r="R10" s="181"/>
-      <c r="S10" s="181"/>
-      <c r="T10" s="181"/>
-      <c r="U10" s="181"/>
-      <c r="V10" s="181"/>
-      <c r="W10" s="181"/>
-      <c r="X10" s="181"/>
-      <c r="Y10" s="181"/>
+      <c r="P10" s="119"/>
+      <c r="Q10" s="119"/>
+      <c r="R10" s="119"/>
+      <c r="S10" s="119"/>
+      <c r="T10" s="119"/>
+      <c r="U10" s="119"/>
+      <c r="V10" s="119"/>
+      <c r="W10" s="119"/>
+      <c r="X10" s="119"/>
+      <c r="Y10" s="119"/>
       <c r="Z10" s="15"/>
-      <c r="AA10" s="178" t="s">
+      <c r="AA10" s="118" t="s">
         <v>45</v>
       </c>
-      <c r="AB10" s="178"/>
+      <c r="AB10" s="118"/>
       <c r="AC10" s="15"/>
-      <c r="AD10" s="178" t="s">
+      <c r="AD10" s="118" t="s">
         <v>46</v>
       </c>
-      <c r="AE10" s="178"/>
+      <c r="AE10" s="118"/>
       <c r="AF10" s="15"/>
-      <c r="AG10" s="178" t="s">
+      <c r="AG10" s="118" t="s">
         <v>47</v>
       </c>
-      <c r="AH10" s="178"/>
+      <c r="AH10" s="118"/>
       <c r="AI10" s="9"/>
       <c r="AJ10" s="85"/>
       <c r="AK10" s="85"/>
@@ -2662,33 +2719,33 @@
     </row>
     <row r="11" spans="1:45" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="16"/>
-      <c r="B11" s="138" t="s">
+      <c r="B11" s="108" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="138"/>
-      <c r="D11" s="138"/>
-      <c r="E11" s="138"/>
-      <c r="F11" s="138"/>
-      <c r="G11" s="138"/>
-      <c r="H11" s="138"/>
-      <c r="I11" s="138"/>
-      <c r="J11" s="138"/>
-      <c r="K11" s="197"/>
-      <c r="L11" s="198"/>
-      <c r="M11" s="198"/>
-      <c r="N11" s="198"/>
-      <c r="O11" s="198"/>
-      <c r="P11" s="198"/>
-      <c r="Q11" s="198"/>
-      <c r="R11" s="198"/>
-      <c r="S11" s="198"/>
-      <c r="T11" s="198"/>
-      <c r="U11" s="198"/>
-      <c r="V11" s="199"/>
-      <c r="W11" s="184" t="s">
+      <c r="C11" s="108"/>
+      <c r="D11" s="108"/>
+      <c r="E11" s="108"/>
+      <c r="F11" s="108"/>
+      <c r="G11" s="108"/>
+      <c r="H11" s="108"/>
+      <c r="I11" s="108"/>
+      <c r="J11" s="108"/>
+      <c r="K11" s="109"/>
+      <c r="L11" s="110"/>
+      <c r="M11" s="110"/>
+      <c r="N11" s="110"/>
+      <c r="O11" s="110"/>
+      <c r="P11" s="110"/>
+      <c r="Q11" s="110"/>
+      <c r="R11" s="110"/>
+      <c r="S11" s="110"/>
+      <c r="T11" s="110"/>
+      <c r="U11" s="110"/>
+      <c r="V11" s="111"/>
+      <c r="W11" s="112" t="s">
         <v>12</v>
       </c>
-      <c r="X11" s="184"/>
+      <c r="X11" s="112"/>
       <c r="Y11" s="64"/>
       <c r="Z11" s="64"/>
       <c r="AA11" s="65"/>
@@ -2733,20 +2790,20 @@
       <c r="H12" s="17"/>
       <c r="I12" s="17"/>
       <c r="J12" s="17"/>
-      <c r="K12" s="196" t="s">
+      <c r="K12" s="105" t="s">
         <v>28</v>
       </c>
-      <c r="L12" s="196"/>
-      <c r="M12" s="196"/>
-      <c r="N12" s="196"/>
-      <c r="O12" s="196"/>
-      <c r="P12" s="196"/>
-      <c r="Q12" s="196"/>
-      <c r="R12" s="196"/>
-      <c r="S12" s="196"/>
-      <c r="T12" s="196"/>
-      <c r="U12" s="196"/>
-      <c r="V12" s="196"/>
+      <c r="L12" s="105"/>
+      <c r="M12" s="105"/>
+      <c r="N12" s="105"/>
+      <c r="O12" s="105"/>
+      <c r="P12" s="105"/>
+      <c r="Q12" s="105"/>
+      <c r="R12" s="105"/>
+      <c r="S12" s="105"/>
+      <c r="T12" s="105"/>
+      <c r="U12" s="105"/>
+      <c r="V12" s="105"/>
       <c r="W12" s="18"/>
       <c r="X12" s="18"/>
       <c r="Y12" s="19"/>
@@ -2840,41 +2897,41 @@
       <c r="A14" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="B14" s="138" t="s">
+      <c r="B14" s="108" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="138"/>
-      <c r="D14" s="138"/>
-      <c r="E14" s="138"/>
-      <c r="F14" s="138"/>
-      <c r="G14" s="138"/>
-      <c r="H14" s="138"/>
-      <c r="I14" s="138"/>
-      <c r="J14" s="138"/>
-      <c r="K14" s="138"/>
-      <c r="L14" s="138"/>
-      <c r="M14" s="100"/>
-      <c r="N14" s="101"/>
-      <c r="O14" s="101"/>
-      <c r="P14" s="101"/>
-      <c r="Q14" s="101"/>
-      <c r="R14" s="101"/>
-      <c r="S14" s="101"/>
-      <c r="T14" s="101"/>
-      <c r="U14" s="101"/>
-      <c r="V14" s="101"/>
-      <c r="W14" s="101"/>
-      <c r="X14" s="101"/>
-      <c r="Y14" s="101"/>
-      <c r="Z14" s="101"/>
-      <c r="AA14" s="101"/>
-      <c r="AB14" s="101"/>
-      <c r="AC14" s="101"/>
-      <c r="AD14" s="101"/>
-      <c r="AE14" s="101"/>
-      <c r="AF14" s="101"/>
-      <c r="AG14" s="101"/>
-      <c r="AH14" s="102"/>
+      <c r="C14" s="108"/>
+      <c r="D14" s="108"/>
+      <c r="E14" s="108"/>
+      <c r="F14" s="108"/>
+      <c r="G14" s="108"/>
+      <c r="H14" s="108"/>
+      <c r="I14" s="108"/>
+      <c r="J14" s="108"/>
+      <c r="K14" s="108"/>
+      <c r="L14" s="108"/>
+      <c r="M14" s="114"/>
+      <c r="N14" s="115"/>
+      <c r="O14" s="115"/>
+      <c r="P14" s="115"/>
+      <c r="Q14" s="115"/>
+      <c r="R14" s="115"/>
+      <c r="S14" s="115"/>
+      <c r="T14" s="115"/>
+      <c r="U14" s="115"/>
+      <c r="V14" s="115"/>
+      <c r="W14" s="115"/>
+      <c r="X14" s="115"/>
+      <c r="Y14" s="115"/>
+      <c r="Z14" s="115"/>
+      <c r="AA14" s="115"/>
+      <c r="AB14" s="115"/>
+      <c r="AC14" s="115"/>
+      <c r="AD14" s="115"/>
+      <c r="AE14" s="115"/>
+      <c r="AF14" s="115"/>
+      <c r="AG14" s="115"/>
+      <c r="AH14" s="116"/>
       <c r="AI14" s="30"/>
       <c r="AJ14" s="85"/>
       <c r="AK14" s="85"/>
@@ -2899,30 +2956,30 @@
     </row>
     <row r="15" spans="1:45" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="16"/>
-      <c r="M15" s="109" t="s">
+      <c r="M15" s="121" t="s">
         <v>88</v>
       </c>
-      <c r="N15" s="109"/>
-      <c r="O15" s="109"/>
-      <c r="P15" s="109"/>
-      <c r="Q15" s="109"/>
-      <c r="R15" s="109"/>
-      <c r="S15" s="109"/>
-      <c r="T15" s="109"/>
-      <c r="U15" s="109"/>
-      <c r="V15" s="109"/>
-      <c r="W15" s="109"/>
-      <c r="X15" s="109"/>
-      <c r="Y15" s="109"/>
-      <c r="Z15" s="109"/>
-      <c r="AA15" s="109"/>
-      <c r="AB15" s="109"/>
-      <c r="AC15" s="109"/>
-      <c r="AD15" s="109"/>
-      <c r="AE15" s="109"/>
-      <c r="AF15" s="109"/>
-      <c r="AG15" s="109"/>
-      <c r="AH15" s="109"/>
+      <c r="N15" s="121"/>
+      <c r="O15" s="121"/>
+      <c r="P15" s="121"/>
+      <c r="Q15" s="121"/>
+      <c r="R15" s="121"/>
+      <c r="S15" s="121"/>
+      <c r="T15" s="121"/>
+      <c r="U15" s="121"/>
+      <c r="V15" s="121"/>
+      <c r="W15" s="121"/>
+      <c r="X15" s="121"/>
+      <c r="Y15" s="121"/>
+      <c r="Z15" s="121"/>
+      <c r="AA15" s="121"/>
+      <c r="AB15" s="121"/>
+      <c r="AC15" s="121"/>
+      <c r="AD15" s="121"/>
+      <c r="AE15" s="121"/>
+      <c r="AF15" s="121"/>
+      <c r="AG15" s="121"/>
+      <c r="AH15" s="121"/>
       <c r="AI15" s="4"/>
       <c r="AJ15" s="85"/>
       <c r="AK15" s="85"/>
@@ -2949,53 +3006,53 @@
       <c r="A16" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="138" t="s">
+      <c r="B16" s="108" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="138"/>
-      <c r="D16" s="138"/>
-      <c r="E16" s="138"/>
-      <c r="F16" s="100"/>
-      <c r="G16" s="101"/>
-      <c r="H16" s="101"/>
-      <c r="I16" s="101"/>
-      <c r="J16" s="102"/>
-      <c r="K16" s="183" t="s">
+      <c r="C16" s="108"/>
+      <c r="D16" s="108"/>
+      <c r="E16" s="108"/>
+      <c r="F16" s="114"/>
+      <c r="G16" s="115"/>
+      <c r="H16" s="115"/>
+      <c r="I16" s="115"/>
+      <c r="J16" s="116"/>
+      <c r="K16" s="122" t="s">
         <v>51</v>
       </c>
-      <c r="L16" s="183"/>
-      <c r="M16" s="183"/>
-      <c r="N16" s="183"/>
-      <c r="O16" s="183"/>
-      <c r="P16" s="183"/>
-      <c r="Q16" s="168"/>
-      <c r="R16" s="169"/>
-      <c r="S16" s="170" t="s">
+      <c r="L16" s="122"/>
+      <c r="M16" s="122"/>
+      <c r="N16" s="122"/>
+      <c r="O16" s="122"/>
+      <c r="P16" s="122"/>
+      <c r="Q16" s="123"/>
+      <c r="R16" s="124"/>
+      <c r="S16" s="125" t="s">
         <v>17</v>
       </c>
-      <c r="T16" s="170"/>
-      <c r="U16" s="177" t="s">
+      <c r="T16" s="125"/>
+      <c r="U16" s="126" t="s">
         <v>30</v>
       </c>
-      <c r="V16" s="177"/>
-      <c r="W16" s="177"/>
-      <c r="X16" s="177"/>
-      <c r="Y16" s="177"/>
-      <c r="Z16" s="173">
+      <c r="V16" s="126"/>
+      <c r="W16" s="126"/>
+      <c r="X16" s="126"/>
+      <c r="Y16" s="126"/>
+      <c r="Z16" s="127">
         <v>0</v>
       </c>
-      <c r="AA16" s="173"/>
-      <c r="AB16" s="184" t="s">
+      <c r="AA16" s="127"/>
+      <c r="AB16" s="112" t="s">
         <v>31</v>
       </c>
-      <c r="AC16" s="184"/>
-      <c r="AD16" s="184"/>
-      <c r="AE16" s="184"/>
-      <c r="AF16" s="184"/>
-      <c r="AG16" s="175">
+      <c r="AC16" s="112"/>
+      <c r="AD16" s="112"/>
+      <c r="AE16" s="112"/>
+      <c r="AF16" s="112"/>
+      <c r="AG16" s="128">
         <v>1</v>
       </c>
-      <c r="AH16" s="175"/>
+      <c r="AH16" s="128"/>
       <c r="AI16" s="4"/>
       <c r="AJ16" s="85"/>
       <c r="AK16" s="85"/>
@@ -3016,41 +3073,41 @@
     </row>
     <row r="17" spans="1:45" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="31"/>
-      <c r="B17" s="176" t="s">
+      <c r="B17" s="130" t="s">
         <v>36</v>
       </c>
-      <c r="C17" s="176"/>
-      <c r="D17" s="176"/>
-      <c r="E17" s="176"/>
-      <c r="F17" s="176"/>
-      <c r="G17" s="176"/>
-      <c r="H17" s="176"/>
-      <c r="I17" s="176"/>
-      <c r="J17" s="176"/>
-      <c r="K17" s="176"/>
-      <c r="L17" s="176"/>
-      <c r="M17" s="176"/>
-      <c r="N17" s="176"/>
-      <c r="O17" s="176"/>
-      <c r="P17" s="176"/>
-      <c r="Q17" s="176"/>
-      <c r="R17" s="176"/>
-      <c r="S17" s="176"/>
-      <c r="T17" s="176"/>
-      <c r="U17" s="176"/>
-      <c r="V17" s="176"/>
-      <c r="W17" s="176"/>
-      <c r="X17" s="176"/>
-      <c r="Y17" s="176"/>
-      <c r="Z17" s="176"/>
-      <c r="AA17" s="176"/>
-      <c r="AB17" s="176"/>
-      <c r="AC17" s="176"/>
-      <c r="AD17" s="176"/>
-      <c r="AE17" s="176"/>
-      <c r="AF17" s="176"/>
-      <c r="AG17" s="176"/>
-      <c r="AH17" s="176"/>
+      <c r="C17" s="130"/>
+      <c r="D17" s="130"/>
+      <c r="E17" s="130"/>
+      <c r="F17" s="130"/>
+      <c r="G17" s="130"/>
+      <c r="H17" s="130"/>
+      <c r="I17" s="130"/>
+      <c r="J17" s="130"/>
+      <c r="K17" s="130"/>
+      <c r="L17" s="130"/>
+      <c r="M17" s="130"/>
+      <c r="N17" s="130"/>
+      <c r="O17" s="130"/>
+      <c r="P17" s="130"/>
+      <c r="Q17" s="130"/>
+      <c r="R17" s="130"/>
+      <c r="S17" s="130"/>
+      <c r="T17" s="130"/>
+      <c r="U17" s="130"/>
+      <c r="V17" s="130"/>
+      <c r="W17" s="130"/>
+      <c r="X17" s="130"/>
+      <c r="Y17" s="130"/>
+      <c r="Z17" s="130"/>
+      <c r="AA17" s="130"/>
+      <c r="AB17" s="130"/>
+      <c r="AC17" s="130"/>
+      <c r="AD17" s="130"/>
+      <c r="AE17" s="130"/>
+      <c r="AF17" s="130"/>
+      <c r="AG17" s="130"/>
+      <c r="AH17" s="130"/>
       <c r="AI17" s="4"/>
       <c r="AJ17" s="85"/>
       <c r="AK17" s="85"/>
@@ -3072,46 +3129,46 @@
     <row r="18" spans="1:45" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="31"/>
       <c r="B18" s="32"/>
-      <c r="C18" s="171" t="s">
+      <c r="C18" s="131" t="s">
         <v>65</v>
       </c>
-      <c r="D18" s="171"/>
-      <c r="E18" s="171"/>
-      <c r="F18" s="171"/>
-      <c r="G18" s="171"/>
-      <c r="H18" s="171"/>
-      <c r="I18" s="171"/>
-      <c r="J18" s="171"/>
-      <c r="K18" s="171" t="s">
+      <c r="D18" s="131"/>
+      <c r="E18" s="131"/>
+      <c r="F18" s="131"/>
+      <c r="G18" s="131"/>
+      <c r="H18" s="131"/>
+      <c r="I18" s="131"/>
+      <c r="J18" s="131"/>
+      <c r="K18" s="131" t="s">
         <v>65</v>
       </c>
-      <c r="L18" s="171"/>
-      <c r="M18" s="171"/>
-      <c r="N18" s="171"/>
-      <c r="O18" s="171"/>
-      <c r="P18" s="171"/>
-      <c r="Q18" s="171"/>
-      <c r="R18" s="171"/>
-      <c r="S18" s="171" t="s">
+      <c r="L18" s="131"/>
+      <c r="M18" s="131"/>
+      <c r="N18" s="131"/>
+      <c r="O18" s="131"/>
+      <c r="P18" s="131"/>
+      <c r="Q18" s="131"/>
+      <c r="R18" s="131"/>
+      <c r="S18" s="131" t="s">
         <v>65</v>
       </c>
-      <c r="T18" s="171"/>
-      <c r="U18" s="171"/>
-      <c r="V18" s="171"/>
-      <c r="W18" s="171"/>
-      <c r="X18" s="171"/>
-      <c r="Y18" s="171"/>
-      <c r="Z18" s="171"/>
-      <c r="AA18" s="171" t="s">
+      <c r="T18" s="131"/>
+      <c r="U18" s="131"/>
+      <c r="V18" s="131"/>
+      <c r="W18" s="131"/>
+      <c r="X18" s="131"/>
+      <c r="Y18" s="131"/>
+      <c r="Z18" s="131"/>
+      <c r="AA18" s="131" t="s">
         <v>65</v>
       </c>
-      <c r="AB18" s="171"/>
-      <c r="AC18" s="171"/>
-      <c r="AD18" s="171"/>
-      <c r="AE18" s="171"/>
-      <c r="AF18" s="171"/>
-      <c r="AG18" s="171"/>
-      <c r="AH18" s="171"/>
+      <c r="AB18" s="131"/>
+      <c r="AC18" s="131"/>
+      <c r="AD18" s="131"/>
+      <c r="AE18" s="131"/>
+      <c r="AF18" s="131"/>
+      <c r="AG18" s="131"/>
+      <c r="AH18" s="131"/>
       <c r="AI18" s="4"/>
       <c r="AJ18" s="85"/>
       <c r="AK18" s="85"/>
@@ -3131,38 +3188,38 @@
     <row r="19" spans="1:45" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="31"/>
       <c r="B19" s="17"/>
-      <c r="C19" s="96"/>
-      <c r="D19" s="103"/>
-      <c r="E19" s="103"/>
-      <c r="F19" s="103"/>
-      <c r="G19" s="103"/>
-      <c r="H19" s="103"/>
-      <c r="I19" s="103"/>
-      <c r="J19" s="97"/>
-      <c r="K19" s="96"/>
-      <c r="L19" s="103"/>
-      <c r="M19" s="103"/>
-      <c r="N19" s="103"/>
-      <c r="O19" s="103"/>
-      <c r="P19" s="103"/>
-      <c r="Q19" s="103"/>
-      <c r="R19" s="97"/>
-      <c r="S19" s="96"/>
-      <c r="T19" s="103"/>
-      <c r="U19" s="103"/>
-      <c r="V19" s="103"/>
-      <c r="W19" s="103"/>
-      <c r="X19" s="103"/>
-      <c r="Y19" s="103"/>
-      <c r="Z19" s="97"/>
-      <c r="AA19" s="96"/>
-      <c r="AB19" s="103"/>
-      <c r="AC19" s="103"/>
-      <c r="AD19" s="103"/>
-      <c r="AE19" s="103"/>
-      <c r="AF19" s="103"/>
-      <c r="AG19" s="103"/>
-      <c r="AH19" s="97"/>
+      <c r="C19" s="106"/>
+      <c r="D19" s="117"/>
+      <c r="E19" s="117"/>
+      <c r="F19" s="117"/>
+      <c r="G19" s="117"/>
+      <c r="H19" s="117"/>
+      <c r="I19" s="117"/>
+      <c r="J19" s="107"/>
+      <c r="K19" s="106"/>
+      <c r="L19" s="117"/>
+      <c r="M19" s="117"/>
+      <c r="N19" s="117"/>
+      <c r="O19" s="117"/>
+      <c r="P19" s="117"/>
+      <c r="Q19" s="117"/>
+      <c r="R19" s="107"/>
+      <c r="S19" s="106"/>
+      <c r="T19" s="117"/>
+      <c r="U19" s="117"/>
+      <c r="V19" s="117"/>
+      <c r="W19" s="117"/>
+      <c r="X19" s="117"/>
+      <c r="Y19" s="117"/>
+      <c r="Z19" s="107"/>
+      <c r="AA19" s="106"/>
+      <c r="AB19" s="117"/>
+      <c r="AC19" s="117"/>
+      <c r="AD19" s="117"/>
+      <c r="AE19" s="117"/>
+      <c r="AF19" s="117"/>
+      <c r="AG19" s="117"/>
+      <c r="AH19" s="107"/>
       <c r="AI19" s="4"/>
       <c r="AJ19" s="85"/>
       <c r="AK19" s="85"/>
@@ -3181,54 +3238,54 @@
     </row>
     <row r="20" spans="1:45" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="31"/>
-      <c r="C20" s="172" t="s">
+      <c r="C20" s="129" t="s">
         <v>18</v>
       </c>
-      <c r="D20" s="172"/>
-      <c r="E20" s="96"/>
-      <c r="F20" s="97"/>
-      <c r="G20" s="172" t="s">
+      <c r="D20" s="129"/>
+      <c r="E20" s="106"/>
+      <c r="F20" s="107"/>
+      <c r="G20" s="129" t="s">
         <v>19</v>
       </c>
-      <c r="H20" s="172"/>
-      <c r="I20" s="96"/>
-      <c r="J20" s="97"/>
-      <c r="K20" s="172" t="s">
+      <c r="H20" s="129"/>
+      <c r="I20" s="106"/>
+      <c r="J20" s="107"/>
+      <c r="K20" s="129" t="s">
         <v>18</v>
       </c>
-      <c r="L20" s="172"/>
-      <c r="M20" s="179"/>
-      <c r="N20" s="180"/>
-      <c r="O20" s="172" t="s">
+      <c r="L20" s="129"/>
+      <c r="M20" s="132"/>
+      <c r="N20" s="133"/>
+      <c r="O20" s="129" t="s">
         <v>19</v>
       </c>
-      <c r="P20" s="172"/>
-      <c r="Q20" s="96"/>
-      <c r="R20" s="97"/>
-      <c r="S20" s="172" t="s">
+      <c r="P20" s="129"/>
+      <c r="Q20" s="106"/>
+      <c r="R20" s="107"/>
+      <c r="S20" s="129" t="s">
         <v>18</v>
       </c>
-      <c r="T20" s="172"/>
-      <c r="U20" s="96"/>
-      <c r="V20" s="97"/>
-      <c r="W20" s="172" t="s">
+      <c r="T20" s="129"/>
+      <c r="U20" s="106"/>
+      <c r="V20" s="107"/>
+      <c r="W20" s="129" t="s">
         <v>19</v>
       </c>
-      <c r="X20" s="172"/>
-      <c r="Y20" s="96"/>
-      <c r="Z20" s="97"/>
-      <c r="AA20" s="172" t="s">
+      <c r="X20" s="129"/>
+      <c r="Y20" s="106"/>
+      <c r="Z20" s="107"/>
+      <c r="AA20" s="129" t="s">
         <v>18</v>
       </c>
-      <c r="AB20" s="172"/>
-      <c r="AC20" s="96"/>
-      <c r="AD20" s="97"/>
-      <c r="AE20" s="172" t="s">
+      <c r="AB20" s="129"/>
+      <c r="AC20" s="106"/>
+      <c r="AD20" s="107"/>
+      <c r="AE20" s="129" t="s">
         <v>19</v>
       </c>
-      <c r="AF20" s="172"/>
-      <c r="AG20" s="96"/>
-      <c r="AH20" s="97"/>
+      <c r="AF20" s="129"/>
+      <c r="AG20" s="106"/>
+      <c r="AH20" s="107"/>
       <c r="AI20" s="4"/>
       <c r="AJ20" s="85"/>
       <c r="AK20" s="85"/>
@@ -3292,41 +3349,41 @@
     </row>
     <row r="22" spans="1:45" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="31"/>
-      <c r="B22" s="99" t="s">
+      <c r="B22" s="136" t="s">
         <v>32</v>
       </c>
-      <c r="C22" s="99"/>
-      <c r="D22" s="99"/>
-      <c r="E22" s="99"/>
-      <c r="F22" s="99"/>
-      <c r="G22" s="99"/>
-      <c r="H22" s="99"/>
-      <c r="I22" s="99"/>
-      <c r="J22" s="99"/>
-      <c r="K22" s="99"/>
+      <c r="C22" s="136"/>
+      <c r="D22" s="136"/>
+      <c r="E22" s="136"/>
+      <c r="F22" s="136"/>
+      <c r="G22" s="136"/>
+      <c r="H22" s="136"/>
+      <c r="I22" s="136"/>
+      <c r="J22" s="136"/>
+      <c r="K22" s="136"/>
       <c r="L22" s="10"/>
-      <c r="M22" s="100"/>
-      <c r="N22" s="101"/>
-      <c r="O22" s="101"/>
-      <c r="P22" s="101"/>
-      <c r="Q22" s="101"/>
-      <c r="R22" s="101"/>
-      <c r="S22" s="101"/>
-      <c r="T22" s="101"/>
-      <c r="U22" s="102"/>
+      <c r="M22" s="114"/>
+      <c r="N22" s="115"/>
+      <c r="O22" s="115"/>
+      <c r="P22" s="115"/>
+      <c r="Q22" s="115"/>
+      <c r="R22" s="115"/>
+      <c r="S22" s="115"/>
+      <c r="T22" s="115"/>
+      <c r="U22" s="116"/>
       <c r="V22" s="70"/>
-      <c r="W22" s="96"/>
-      <c r="X22" s="97"/>
+      <c r="W22" s="106"/>
+      <c r="X22" s="107"/>
       <c r="Y22" s="70"/>
-      <c r="Z22" s="96"/>
-      <c r="AA22" s="97"/>
+      <c r="Z22" s="106"/>
+      <c r="AA22" s="107"/>
       <c r="AB22" s="74"/>
-      <c r="AC22" s="96"/>
-      <c r="AD22" s="97"/>
+      <c r="AC22" s="106"/>
+      <c r="AD22" s="107"/>
       <c r="AE22" s="74"/>
-      <c r="AF22" s="96"/>
-      <c r="AG22" s="103"/>
-      <c r="AH22" s="97"/>
+      <c r="AF22" s="106"/>
+      <c r="AG22" s="117"/>
+      <c r="AH22" s="107"/>
       <c r="AJ22" s="85"/>
       <c r="AK22" s="85"/>
       <c r="AL22" s="85"/>
@@ -3365,26 +3422,26 @@
       <c r="S23" s="34"/>
       <c r="U23" s="34"/>
       <c r="V23" s="34"/>
-      <c r="W23" s="178" t="s">
+      <c r="W23" s="118" t="s">
         <v>45</v>
       </c>
-      <c r="X23" s="178"/>
+      <c r="X23" s="118"/>
       <c r="Y23" s="35"/>
-      <c r="Z23" s="178" t="s">
+      <c r="Z23" s="118" t="s">
         <v>46</v>
       </c>
-      <c r="AA23" s="178"/>
+      <c r="AA23" s="118"/>
       <c r="AB23" s="35"/>
-      <c r="AC23" s="178" t="s">
+      <c r="AC23" s="118" t="s">
         <v>47</v>
       </c>
-      <c r="AD23" s="178"/>
+      <c r="AD23" s="118"/>
       <c r="AE23" s="35"/>
-      <c r="AF23" s="178" t="s">
+      <c r="AF23" s="118" t="s">
         <v>52</v>
       </c>
-      <c r="AG23" s="178"/>
-      <c r="AH23" s="178"/>
+      <c r="AG23" s="118"/>
+      <c r="AH23" s="118"/>
       <c r="AJ23" s="85"/>
       <c r="AK23" s="85"/>
       <c r="AL23" s="85"/>
@@ -3402,41 +3459,41 @@
     </row>
     <row r="24" spans="1:45" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="31"/>
-      <c r="B24" s="99" t="s">
+      <c r="B24" s="136" t="s">
         <v>33</v>
       </c>
-      <c r="C24" s="99"/>
-      <c r="D24" s="99"/>
-      <c r="E24" s="99"/>
-      <c r="F24" s="99"/>
-      <c r="G24" s="99"/>
-      <c r="H24" s="99"/>
-      <c r="I24" s="99"/>
-      <c r="J24" s="99"/>
-      <c r="K24" s="99"/>
+      <c r="C24" s="136"/>
+      <c r="D24" s="136"/>
+      <c r="E24" s="136"/>
+      <c r="F24" s="136"/>
+      <c r="G24" s="136"/>
+      <c r="H24" s="136"/>
+      <c r="I24" s="136"/>
+      <c r="J24" s="136"/>
+      <c r="K24" s="136"/>
       <c r="L24" s="10"/>
-      <c r="M24" s="100"/>
-      <c r="N24" s="101"/>
-      <c r="O24" s="101"/>
-      <c r="P24" s="101"/>
-      <c r="Q24" s="101"/>
-      <c r="R24" s="101"/>
-      <c r="S24" s="101"/>
-      <c r="T24" s="101"/>
-      <c r="U24" s="102"/>
+      <c r="M24" s="114"/>
+      <c r="N24" s="115"/>
+      <c r="O24" s="115"/>
+      <c r="P24" s="115"/>
+      <c r="Q24" s="115"/>
+      <c r="R24" s="115"/>
+      <c r="S24" s="115"/>
+      <c r="T24" s="115"/>
+      <c r="U24" s="116"/>
       <c r="V24" s="75"/>
-      <c r="W24" s="96"/>
-      <c r="X24" s="97"/>
+      <c r="W24" s="106"/>
+      <c r="X24" s="107"/>
       <c r="Y24" s="70"/>
-      <c r="Z24" s="96"/>
-      <c r="AA24" s="97"/>
+      <c r="Z24" s="106"/>
+      <c r="AA24" s="107"/>
       <c r="AB24" s="74"/>
-      <c r="AC24" s="96"/>
-      <c r="AD24" s="97"/>
+      <c r="AC24" s="106"/>
+      <c r="AD24" s="107"/>
       <c r="AE24" s="74"/>
-      <c r="AF24" s="96"/>
-      <c r="AG24" s="103"/>
-      <c r="AH24" s="97"/>
+      <c r="AF24" s="106"/>
+      <c r="AG24" s="117"/>
+      <c r="AH24" s="107"/>
       <c r="AJ24" s="85"/>
       <c r="AK24" s="85"/>
       <c r="AL24" s="85"/>
@@ -3475,26 +3532,26 @@
       <c r="S25" s="34"/>
       <c r="U25" s="34"/>
       <c r="V25" s="34"/>
-      <c r="W25" s="178" t="s">
+      <c r="W25" s="118" t="s">
         <v>45</v>
       </c>
-      <c r="X25" s="178"/>
+      <c r="X25" s="118"/>
       <c r="Y25" s="35"/>
-      <c r="Z25" s="178" t="s">
+      <c r="Z25" s="118" t="s">
         <v>46</v>
       </c>
-      <c r="AA25" s="178"/>
+      <c r="AA25" s="118"/>
       <c r="AB25" s="35"/>
-      <c r="AC25" s="178" t="s">
+      <c r="AC25" s="118" t="s">
         <v>47</v>
       </c>
-      <c r="AD25" s="178"/>
+      <c r="AD25" s="118"/>
       <c r="AE25" s="35"/>
-      <c r="AF25" s="178" t="s">
+      <c r="AF25" s="118" t="s">
         <v>52</v>
       </c>
-      <c r="AG25" s="178"/>
-      <c r="AH25" s="178"/>
+      <c r="AG25" s="118"/>
+      <c r="AH25" s="118"/>
       <c r="AJ25" s="85"/>
       <c r="AK25" s="85"/>
       <c r="AL25" s="85"/>
@@ -3565,53 +3622,53 @@
       <c r="A27" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="B27" s="138" t="s">
+      <c r="B27" s="108" t="s">
         <v>29</v>
       </c>
-      <c r="C27" s="138"/>
-      <c r="D27" s="138"/>
-      <c r="E27" s="138"/>
-      <c r="F27" s="100"/>
-      <c r="G27" s="101"/>
-      <c r="H27" s="101"/>
-      <c r="I27" s="101"/>
-      <c r="J27" s="102"/>
-      <c r="K27" s="172" t="s">
+      <c r="C27" s="108"/>
+      <c r="D27" s="108"/>
+      <c r="E27" s="108"/>
+      <c r="F27" s="114"/>
+      <c r="G27" s="115"/>
+      <c r="H27" s="115"/>
+      <c r="I27" s="115"/>
+      <c r="J27" s="116"/>
+      <c r="K27" s="129" t="s">
         <v>76</v>
       </c>
-      <c r="L27" s="172"/>
-      <c r="M27" s="172"/>
-      <c r="N27" s="172"/>
-      <c r="O27" s="172"/>
-      <c r="P27" s="172"/>
-      <c r="Q27" s="168"/>
-      <c r="R27" s="169"/>
-      <c r="S27" s="170" t="s">
+      <c r="L27" s="129"/>
+      <c r="M27" s="129"/>
+      <c r="N27" s="129"/>
+      <c r="O27" s="129"/>
+      <c r="P27" s="129"/>
+      <c r="Q27" s="123"/>
+      <c r="R27" s="124"/>
+      <c r="S27" s="125" t="s">
         <v>17</v>
       </c>
-      <c r="T27" s="170"/>
-      <c r="U27" s="177" t="s">
+      <c r="T27" s="125"/>
+      <c r="U27" s="126" t="s">
         <v>30</v>
       </c>
-      <c r="V27" s="177"/>
-      <c r="W27" s="177"/>
-      <c r="X27" s="177"/>
-      <c r="Y27" s="177"/>
-      <c r="Z27" s="173">
+      <c r="V27" s="126"/>
+      <c r="W27" s="126"/>
+      <c r="X27" s="126"/>
+      <c r="Y27" s="126"/>
+      <c r="Z27" s="127">
         <v>0</v>
       </c>
-      <c r="AA27" s="173"/>
-      <c r="AB27" s="174" t="s">
+      <c r="AA27" s="127"/>
+      <c r="AB27" s="137" t="s">
         <v>31</v>
       </c>
-      <c r="AC27" s="174"/>
-      <c r="AD27" s="174"/>
-      <c r="AE27" s="174"/>
-      <c r="AF27" s="174"/>
-      <c r="AG27" s="175">
+      <c r="AC27" s="137"/>
+      <c r="AD27" s="137"/>
+      <c r="AE27" s="137"/>
+      <c r="AF27" s="137"/>
+      <c r="AG27" s="128">
         <v>1</v>
       </c>
-      <c r="AH27" s="175"/>
+      <c r="AH27" s="128"/>
       <c r="AI27" s="4"/>
       <c r="AJ27" s="85"/>
       <c r="AK27" s="85"/>
@@ -3630,41 +3687,41 @@
     </row>
     <row r="28" spans="1:45" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="16"/>
-      <c r="B28" s="176" t="s">
+      <c r="B28" s="130" t="s">
         <v>36</v>
       </c>
-      <c r="C28" s="176"/>
-      <c r="D28" s="176"/>
-      <c r="E28" s="176"/>
-      <c r="F28" s="176"/>
-      <c r="G28" s="176"/>
-      <c r="H28" s="176"/>
-      <c r="I28" s="176"/>
-      <c r="J28" s="176"/>
-      <c r="K28" s="176"/>
-      <c r="L28" s="176"/>
-      <c r="M28" s="176"/>
-      <c r="N28" s="176"/>
-      <c r="O28" s="176"/>
-      <c r="P28" s="176"/>
-      <c r="Q28" s="176"/>
-      <c r="R28" s="176"/>
-      <c r="S28" s="176"/>
-      <c r="T28" s="176"/>
-      <c r="U28" s="176"/>
-      <c r="V28" s="176"/>
-      <c r="W28" s="176"/>
-      <c r="X28" s="176"/>
-      <c r="Y28" s="176"/>
-      <c r="Z28" s="176"/>
-      <c r="AA28" s="176"/>
-      <c r="AB28" s="176"/>
-      <c r="AC28" s="176"/>
-      <c r="AD28" s="176"/>
-      <c r="AE28" s="176"/>
-      <c r="AF28" s="176"/>
-      <c r="AG28" s="176"/>
-      <c r="AH28" s="176"/>
+      <c r="C28" s="130"/>
+      <c r="D28" s="130"/>
+      <c r="E28" s="130"/>
+      <c r="F28" s="130"/>
+      <c r="G28" s="130"/>
+      <c r="H28" s="130"/>
+      <c r="I28" s="130"/>
+      <c r="J28" s="130"/>
+      <c r="K28" s="130"/>
+      <c r="L28" s="130"/>
+      <c r="M28" s="130"/>
+      <c r="N28" s="130"/>
+      <c r="O28" s="130"/>
+      <c r="P28" s="130"/>
+      <c r="Q28" s="130"/>
+      <c r="R28" s="130"/>
+      <c r="S28" s="130"/>
+      <c r="T28" s="130"/>
+      <c r="U28" s="130"/>
+      <c r="V28" s="130"/>
+      <c r="W28" s="130"/>
+      <c r="X28" s="130"/>
+      <c r="Y28" s="130"/>
+      <c r="Z28" s="130"/>
+      <c r="AA28" s="130"/>
+      <c r="AB28" s="130"/>
+      <c r="AC28" s="130"/>
+      <c r="AD28" s="130"/>
+      <c r="AE28" s="130"/>
+      <c r="AF28" s="130"/>
+      <c r="AG28" s="130"/>
+      <c r="AH28" s="130"/>
       <c r="AI28" s="4"/>
       <c r="AJ28" s="85"/>
       <c r="AK28" s="85"/>
@@ -3684,46 +3741,46 @@
     <row r="29" spans="1:45" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="16"/>
       <c r="B29" s="63"/>
-      <c r="C29" s="171" t="s">
+      <c r="C29" s="131" t="s">
         <v>65</v>
       </c>
-      <c r="D29" s="171"/>
-      <c r="E29" s="171"/>
-      <c r="F29" s="171"/>
-      <c r="G29" s="171"/>
-      <c r="H29" s="171"/>
-      <c r="I29" s="171"/>
-      <c r="J29" s="171"/>
-      <c r="K29" s="171" t="s">
+      <c r="D29" s="131"/>
+      <c r="E29" s="131"/>
+      <c r="F29" s="131"/>
+      <c r="G29" s="131"/>
+      <c r="H29" s="131"/>
+      <c r="I29" s="131"/>
+      <c r="J29" s="131"/>
+      <c r="K29" s="131" t="s">
         <v>65</v>
       </c>
-      <c r="L29" s="171"/>
-      <c r="M29" s="171"/>
-      <c r="N29" s="171"/>
-      <c r="O29" s="171"/>
-      <c r="P29" s="171"/>
-      <c r="Q29" s="171"/>
-      <c r="R29" s="171"/>
-      <c r="S29" s="171" t="s">
+      <c r="L29" s="131"/>
+      <c r="M29" s="131"/>
+      <c r="N29" s="131"/>
+      <c r="O29" s="131"/>
+      <c r="P29" s="131"/>
+      <c r="Q29" s="131"/>
+      <c r="R29" s="131"/>
+      <c r="S29" s="131" t="s">
         <v>65</v>
       </c>
-      <c r="T29" s="171"/>
-      <c r="U29" s="171"/>
-      <c r="V29" s="171"/>
-      <c r="W29" s="171"/>
-      <c r="X29" s="171"/>
-      <c r="Y29" s="171"/>
-      <c r="Z29" s="171"/>
-      <c r="AA29" s="171" t="s">
+      <c r="T29" s="131"/>
+      <c r="U29" s="131"/>
+      <c r="V29" s="131"/>
+      <c r="W29" s="131"/>
+      <c r="X29" s="131"/>
+      <c r="Y29" s="131"/>
+      <c r="Z29" s="131"/>
+      <c r="AA29" s="131" t="s">
         <v>65</v>
       </c>
-      <c r="AB29" s="171"/>
-      <c r="AC29" s="171"/>
-      <c r="AD29" s="171"/>
-      <c r="AE29" s="171"/>
-      <c r="AF29" s="171"/>
-      <c r="AG29" s="171"/>
-      <c r="AH29" s="171"/>
+      <c r="AB29" s="131"/>
+      <c r="AC29" s="131"/>
+      <c r="AD29" s="131"/>
+      <c r="AE29" s="131"/>
+      <c r="AF29" s="131"/>
+      <c r="AG29" s="131"/>
+      <c r="AH29" s="131"/>
       <c r="AI29" s="4"/>
       <c r="AJ29" s="85"/>
       <c r="AK29" s="85"/>
@@ -3743,38 +3800,38 @@
     <row r="30" spans="1:45" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="16"/>
       <c r="B30" s="17"/>
-      <c r="C30" s="96"/>
-      <c r="D30" s="103"/>
-      <c r="E30" s="103"/>
-      <c r="F30" s="103"/>
-      <c r="G30" s="103"/>
-      <c r="H30" s="103"/>
-      <c r="I30" s="103"/>
-      <c r="J30" s="97"/>
-      <c r="K30" s="96"/>
-      <c r="L30" s="103"/>
-      <c r="M30" s="103"/>
-      <c r="N30" s="103"/>
-      <c r="O30" s="103"/>
-      <c r="P30" s="103"/>
-      <c r="Q30" s="103"/>
-      <c r="R30" s="97"/>
-      <c r="S30" s="96"/>
-      <c r="T30" s="103"/>
-      <c r="U30" s="103"/>
-      <c r="V30" s="103"/>
-      <c r="W30" s="103"/>
-      <c r="X30" s="103"/>
-      <c r="Y30" s="103"/>
-      <c r="Z30" s="97"/>
-      <c r="AA30" s="96"/>
-      <c r="AB30" s="103"/>
-      <c r="AC30" s="103"/>
-      <c r="AD30" s="103"/>
-      <c r="AE30" s="103"/>
-      <c r="AF30" s="103"/>
-      <c r="AG30" s="103"/>
-      <c r="AH30" s="97"/>
+      <c r="C30" s="106"/>
+      <c r="D30" s="117"/>
+      <c r="E30" s="117"/>
+      <c r="F30" s="117"/>
+      <c r="G30" s="117"/>
+      <c r="H30" s="117"/>
+      <c r="I30" s="117"/>
+      <c r="J30" s="107"/>
+      <c r="K30" s="106"/>
+      <c r="L30" s="117"/>
+      <c r="M30" s="117"/>
+      <c r="N30" s="117"/>
+      <c r="O30" s="117"/>
+      <c r="P30" s="117"/>
+      <c r="Q30" s="117"/>
+      <c r="R30" s="107"/>
+      <c r="S30" s="106"/>
+      <c r="T30" s="117"/>
+      <c r="U30" s="117"/>
+      <c r="V30" s="117"/>
+      <c r="W30" s="117"/>
+      <c r="X30" s="117"/>
+      <c r="Y30" s="117"/>
+      <c r="Z30" s="107"/>
+      <c r="AA30" s="106"/>
+      <c r="AB30" s="117"/>
+      <c r="AC30" s="117"/>
+      <c r="AD30" s="117"/>
+      <c r="AE30" s="117"/>
+      <c r="AF30" s="117"/>
+      <c r="AG30" s="117"/>
+      <c r="AH30" s="107"/>
       <c r="AI30" s="4"/>
       <c r="AJ30" s="85"/>
       <c r="AK30" s="85"/>
@@ -3793,54 +3850,54 @@
     </row>
     <row r="31" spans="1:45" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="16"/>
-      <c r="C31" s="94" t="s">
+      <c r="C31" s="200" t="s">
         <v>18</v>
       </c>
-      <c r="D31" s="95"/>
-      <c r="E31" s="96"/>
-      <c r="F31" s="97"/>
-      <c r="G31" s="98" t="s">
+      <c r="D31" s="135"/>
+      <c r="E31" s="106"/>
+      <c r="F31" s="107"/>
+      <c r="G31" s="134" t="s">
         <v>19</v>
       </c>
-      <c r="H31" s="95"/>
-      <c r="I31" s="96"/>
-      <c r="J31" s="97"/>
-      <c r="K31" s="98" t="s">
+      <c r="H31" s="135"/>
+      <c r="I31" s="106"/>
+      <c r="J31" s="107"/>
+      <c r="K31" s="134" t="s">
         <v>18</v>
       </c>
-      <c r="L31" s="95"/>
-      <c r="M31" s="96"/>
-      <c r="N31" s="97"/>
-      <c r="O31" s="98" t="s">
+      <c r="L31" s="135"/>
+      <c r="M31" s="106"/>
+      <c r="N31" s="107"/>
+      <c r="O31" s="134" t="s">
         <v>19</v>
       </c>
-      <c r="P31" s="95"/>
-      <c r="Q31" s="96"/>
-      <c r="R31" s="97"/>
-      <c r="S31" s="98" t="s">
+      <c r="P31" s="135"/>
+      <c r="Q31" s="106"/>
+      <c r="R31" s="107"/>
+      <c r="S31" s="134" t="s">
         <v>18</v>
       </c>
-      <c r="T31" s="95"/>
-      <c r="U31" s="96"/>
-      <c r="V31" s="97"/>
-      <c r="W31" s="98" t="s">
+      <c r="T31" s="135"/>
+      <c r="U31" s="106"/>
+      <c r="V31" s="107"/>
+      <c r="W31" s="134" t="s">
         <v>19</v>
       </c>
-      <c r="X31" s="95"/>
-      <c r="Y31" s="96"/>
-      <c r="Z31" s="97"/>
-      <c r="AA31" s="98" t="s">
+      <c r="X31" s="135"/>
+      <c r="Y31" s="106"/>
+      <c r="Z31" s="107"/>
+      <c r="AA31" s="134" t="s">
         <v>18</v>
       </c>
-      <c r="AB31" s="95"/>
-      <c r="AC31" s="96"/>
-      <c r="AD31" s="97"/>
-      <c r="AE31" s="98" t="s">
+      <c r="AB31" s="135"/>
+      <c r="AC31" s="106"/>
+      <c r="AD31" s="107"/>
+      <c r="AE31" s="134" t="s">
         <v>19</v>
       </c>
-      <c r="AF31" s="95"/>
-      <c r="AG31" s="96"/>
-      <c r="AH31" s="97"/>
+      <c r="AF31" s="135"/>
+      <c r="AG31" s="106"/>
+      <c r="AH31" s="107"/>
       <c r="AI31" s="4"/>
       <c r="AJ31" s="85"/>
       <c r="AK31" s="85"/>
@@ -3904,41 +3961,41 @@
     </row>
     <row r="33" spans="1:45" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="31"/>
-      <c r="B33" s="99" t="s">
+      <c r="B33" s="136" t="s">
         <v>32</v>
       </c>
-      <c r="C33" s="99"/>
-      <c r="D33" s="99"/>
-      <c r="E33" s="99"/>
-      <c r="F33" s="99"/>
-      <c r="G33" s="99"/>
-      <c r="H33" s="99"/>
-      <c r="I33" s="99"/>
-      <c r="J33" s="99"/>
-      <c r="K33" s="99"/>
+      <c r="C33" s="136"/>
+      <c r="D33" s="136"/>
+      <c r="E33" s="136"/>
+      <c r="F33" s="136"/>
+      <c r="G33" s="136"/>
+      <c r="H33" s="136"/>
+      <c r="I33" s="136"/>
+      <c r="J33" s="136"/>
+      <c r="K33" s="136"/>
       <c r="L33" s="10"/>
-      <c r="M33" s="100"/>
-      <c r="N33" s="101"/>
-      <c r="O33" s="101"/>
-      <c r="P33" s="101"/>
-      <c r="Q33" s="101"/>
-      <c r="R33" s="101"/>
-      <c r="S33" s="101"/>
-      <c r="T33" s="101"/>
-      <c r="U33" s="102"/>
+      <c r="M33" s="114"/>
+      <c r="N33" s="115"/>
+      <c r="O33" s="115"/>
+      <c r="P33" s="115"/>
+      <c r="Q33" s="115"/>
+      <c r="R33" s="115"/>
+      <c r="S33" s="115"/>
+      <c r="T33" s="115"/>
+      <c r="U33" s="116"/>
       <c r="V33" s="70"/>
-      <c r="W33" s="96"/>
-      <c r="X33" s="97"/>
+      <c r="W33" s="106"/>
+      <c r="X33" s="107"/>
       <c r="Y33" s="70"/>
-      <c r="Z33" s="96"/>
-      <c r="AA33" s="97"/>
+      <c r="Z33" s="106"/>
+      <c r="AA33" s="107"/>
       <c r="AB33" s="74"/>
-      <c r="AC33" s="96"/>
-      <c r="AD33" s="97"/>
+      <c r="AC33" s="106"/>
+      <c r="AD33" s="107"/>
       <c r="AE33" s="74"/>
-      <c r="AF33" s="96"/>
-      <c r="AG33" s="103"/>
-      <c r="AH33" s="97"/>
+      <c r="AF33" s="106"/>
+      <c r="AG33" s="117"/>
+      <c r="AH33" s="107"/>
       <c r="AJ33" s="85"/>
       <c r="AK33" s="85"/>
       <c r="AL33" s="85"/>
@@ -3977,26 +4034,26 @@
       <c r="S34" s="34"/>
       <c r="U34" s="34"/>
       <c r="V34" s="34"/>
-      <c r="W34" s="104" t="s">
+      <c r="W34" s="194" t="s">
         <v>45</v>
       </c>
-      <c r="X34" s="104"/>
+      <c r="X34" s="194"/>
       <c r="Y34" s="35"/>
-      <c r="Z34" s="104" t="s">
+      <c r="Z34" s="194" t="s">
         <v>46</v>
       </c>
-      <c r="AA34" s="104"/>
+      <c r="AA34" s="194"/>
       <c r="AB34" s="35"/>
-      <c r="AC34" s="104" t="s">
+      <c r="AC34" s="194" t="s">
         <v>47</v>
       </c>
-      <c r="AD34" s="104"/>
+      <c r="AD34" s="194"/>
       <c r="AE34" s="35"/>
-      <c r="AF34" s="104" t="s">
+      <c r="AF34" s="194" t="s">
         <v>52</v>
       </c>
-      <c r="AG34" s="104"/>
-      <c r="AH34" s="104"/>
+      <c r="AG34" s="194"/>
+      <c r="AH34" s="194"/>
       <c r="AJ34" s="85"/>
       <c r="AK34" s="85"/>
       <c r="AL34" s="85"/>
@@ -4014,41 +4071,41 @@
     </row>
     <row r="35" spans="1:45" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="31"/>
-      <c r="B35" s="99" t="s">
+      <c r="B35" s="136" t="s">
         <v>33</v>
       </c>
-      <c r="C35" s="99"/>
-      <c r="D35" s="99"/>
-      <c r="E35" s="99"/>
-      <c r="F35" s="99"/>
-      <c r="G35" s="99"/>
-      <c r="H35" s="99"/>
-      <c r="I35" s="99"/>
-      <c r="J35" s="99"/>
-      <c r="K35" s="99"/>
+      <c r="C35" s="136"/>
+      <c r="D35" s="136"/>
+      <c r="E35" s="136"/>
+      <c r="F35" s="136"/>
+      <c r="G35" s="136"/>
+      <c r="H35" s="136"/>
+      <c r="I35" s="136"/>
+      <c r="J35" s="136"/>
+      <c r="K35" s="136"/>
       <c r="L35" s="10"/>
-      <c r="M35" s="100"/>
-      <c r="N35" s="101"/>
-      <c r="O35" s="101"/>
-      <c r="P35" s="101"/>
-      <c r="Q35" s="101"/>
-      <c r="R35" s="101"/>
-      <c r="S35" s="101"/>
-      <c r="T35" s="101"/>
-      <c r="U35" s="102"/>
+      <c r="M35" s="114"/>
+      <c r="N35" s="115"/>
+      <c r="O35" s="115"/>
+      <c r="P35" s="115"/>
+      <c r="Q35" s="115"/>
+      <c r="R35" s="115"/>
+      <c r="S35" s="115"/>
+      <c r="T35" s="115"/>
+      <c r="U35" s="116"/>
       <c r="V35" s="70"/>
-      <c r="W35" s="96"/>
-      <c r="X35" s="97"/>
+      <c r="W35" s="106"/>
+      <c r="X35" s="107"/>
       <c r="Y35" s="70"/>
-      <c r="Z35" s="96"/>
-      <c r="AA35" s="97"/>
+      <c r="Z35" s="106"/>
+      <c r="AA35" s="107"/>
       <c r="AB35" s="74"/>
-      <c r="AC35" s="96"/>
-      <c r="AD35" s="97"/>
+      <c r="AC35" s="106"/>
+      <c r="AD35" s="107"/>
       <c r="AE35" s="74"/>
-      <c r="AF35" s="96"/>
-      <c r="AG35" s="103"/>
-      <c r="AH35" s="97"/>
+      <c r="AF35" s="106"/>
+      <c r="AG35" s="117"/>
+      <c r="AH35" s="107"/>
       <c r="AJ35" s="85"/>
       <c r="AK35" s="85"/>
       <c r="AL35" s="85"/>
@@ -4087,26 +4144,26 @@
       <c r="S36" s="34"/>
       <c r="U36" s="34"/>
       <c r="V36" s="34"/>
-      <c r="W36" s="111" t="s">
+      <c r="W36" s="187" t="s">
         <v>45</v>
       </c>
-      <c r="X36" s="111"/>
+      <c r="X36" s="187"/>
       <c r="Y36" s="35"/>
-      <c r="Z36" s="111" t="s">
+      <c r="Z36" s="187" t="s">
         <v>46</v>
       </c>
-      <c r="AA36" s="111"/>
+      <c r="AA36" s="187"/>
       <c r="AB36" s="35"/>
-      <c r="AC36" s="111" t="s">
+      <c r="AC36" s="187" t="s">
         <v>47</v>
       </c>
-      <c r="AD36" s="111"/>
+      <c r="AD36" s="187"/>
       <c r="AE36" s="35"/>
-      <c r="AF36" s="111" t="s">
+      <c r="AF36" s="187" t="s">
         <v>52</v>
       </c>
-      <c r="AG36" s="111"/>
-      <c r="AH36" s="111"/>
+      <c r="AG36" s="187"/>
+      <c r="AH36" s="187"/>
       <c r="AJ36" s="85"/>
       <c r="AK36" s="85"/>
       <c r="AL36" s="85"/>
@@ -4124,41 +4181,41 @@
     </row>
     <row r="37" spans="1:45" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="37"/>
-      <c r="B37" s="105" t="s">
+      <c r="B37" s="195" t="s">
         <v>55</v>
       </c>
-      <c r="C37" s="105"/>
-      <c r="D37" s="105"/>
-      <c r="E37" s="105"/>
-      <c r="F37" s="105"/>
-      <c r="G37" s="105"/>
-      <c r="H37" s="105"/>
-      <c r="I37" s="105"/>
-      <c r="J37" s="105"/>
-      <c r="K37" s="105"/>
-      <c r="L37" s="105"/>
-      <c r="M37" s="105"/>
-      <c r="N37" s="105"/>
-      <c r="O37" s="105"/>
-      <c r="P37" s="105"/>
-      <c r="Q37" s="105"/>
-      <c r="R37" s="105"/>
-      <c r="S37" s="105"/>
-      <c r="T37" s="105"/>
-      <c r="U37" s="105"/>
-      <c r="V37" s="105"/>
-      <c r="W37" s="105"/>
-      <c r="X37" s="105"/>
-      <c r="Y37" s="105"/>
-      <c r="Z37" s="105"/>
-      <c r="AA37" s="105"/>
-      <c r="AB37" s="105"/>
-      <c r="AC37" s="105"/>
-      <c r="AD37" s="105"/>
-      <c r="AE37" s="105"/>
-      <c r="AF37" s="105"/>
-      <c r="AG37" s="105"/>
-      <c r="AH37" s="105"/>
+      <c r="C37" s="195"/>
+      <c r="D37" s="195"/>
+      <c r="E37" s="195"/>
+      <c r="F37" s="195"/>
+      <c r="G37" s="195"/>
+      <c r="H37" s="195"/>
+      <c r="I37" s="195"/>
+      <c r="J37" s="195"/>
+      <c r="K37" s="195"/>
+      <c r="L37" s="195"/>
+      <c r="M37" s="195"/>
+      <c r="N37" s="195"/>
+      <c r="O37" s="195"/>
+      <c r="P37" s="195"/>
+      <c r="Q37" s="195"/>
+      <c r="R37" s="195"/>
+      <c r="S37" s="195"/>
+      <c r="T37" s="195"/>
+      <c r="U37" s="195"/>
+      <c r="V37" s="195"/>
+      <c r="W37" s="195"/>
+      <c r="X37" s="195"/>
+      <c r="Y37" s="195"/>
+      <c r="Z37" s="195"/>
+      <c r="AA37" s="195"/>
+      <c r="AB37" s="195"/>
+      <c r="AC37" s="195"/>
+      <c r="AD37" s="195"/>
+      <c r="AE37" s="195"/>
+      <c r="AF37" s="195"/>
+      <c r="AG37" s="195"/>
+      <c r="AH37" s="195"/>
       <c r="AI37" s="38"/>
       <c r="AJ37" s="85"/>
       <c r="AK37" s="85"/>
@@ -4225,33 +4282,33 @@
       <c r="A39" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="B39" s="106" t="s">
+      <c r="B39" s="196" t="s">
         <v>9</v>
       </c>
-      <c r="C39" s="106"/>
-      <c r="D39" s="106"/>
-      <c r="E39" s="106"/>
-      <c r="F39" s="106"/>
-      <c r="G39" s="106"/>
-      <c r="H39" s="106"/>
-      <c r="I39" s="107"/>
-      <c r="J39" s="96"/>
-      <c r="K39" s="103"/>
-      <c r="L39" s="103"/>
-      <c r="M39" s="103"/>
-      <c r="N39" s="103"/>
-      <c r="O39" s="103"/>
-      <c r="P39" s="103"/>
-      <c r="Q39" s="103"/>
-      <c r="R39" s="103"/>
-      <c r="S39" s="103"/>
-      <c r="T39" s="103"/>
-      <c r="U39" s="103"/>
-      <c r="V39" s="97"/>
-      <c r="W39" s="112" t="s">
+      <c r="C39" s="196"/>
+      <c r="D39" s="196"/>
+      <c r="E39" s="196"/>
+      <c r="F39" s="196"/>
+      <c r="G39" s="196"/>
+      <c r="H39" s="196"/>
+      <c r="I39" s="197"/>
+      <c r="J39" s="106"/>
+      <c r="K39" s="117"/>
+      <c r="L39" s="117"/>
+      <c r="M39" s="117"/>
+      <c r="N39" s="117"/>
+      <c r="O39" s="117"/>
+      <c r="P39" s="117"/>
+      <c r="Q39" s="117"/>
+      <c r="R39" s="117"/>
+      <c r="S39" s="117"/>
+      <c r="T39" s="117"/>
+      <c r="U39" s="117"/>
+      <c r="V39" s="107"/>
+      <c r="W39" s="198" t="s">
         <v>12</v>
       </c>
-      <c r="X39" s="113"/>
+      <c r="X39" s="199"/>
       <c r="Y39" s="64"/>
       <c r="Z39" s="64"/>
       <c r="AA39" s="65"/>
@@ -4274,7 +4331,7 @@
       <c r="AR39" s="85"/>
       <c r="AS39" s="85"/>
     </row>
-    <row r="40" spans="1:45" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:45" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="40"/>
       <c r="B40" s="41"/>
       <c r="C40" s="41"/>
@@ -4284,33 +4341,35 @@
       <c r="G40" s="42"/>
       <c r="H40" s="42"/>
       <c r="I40" s="42"/>
-      <c r="J40" s="110" t="s">
+      <c r="J40" s="186" t="s">
         <v>28</v>
       </c>
-      <c r="K40" s="110"/>
-      <c r="L40" s="110"/>
-      <c r="M40" s="110"/>
-      <c r="N40" s="110"/>
-      <c r="O40" s="110"/>
-      <c r="P40" s="110"/>
-      <c r="Q40" s="110"/>
-      <c r="R40" s="110"/>
-      <c r="S40" s="110"/>
-      <c r="T40" s="110"/>
-      <c r="U40" s="110"/>
-      <c r="V40" s="110"/>
-      <c r="W40" s="42"/>
-      <c r="X40" s="42"/>
-      <c r="Y40" s="42"/>
-      <c r="Z40" s="42"/>
-      <c r="AA40" s="42"/>
-      <c r="AB40" s="42"/>
-      <c r="AC40" s="42"/>
-      <c r="AD40" s="42"/>
-      <c r="AE40" s="42"/>
-      <c r="AF40" s="42"/>
-      <c r="AG40" s="42"/>
-      <c r="AH40" s="42"/>
+      <c r="K40" s="186"/>
+      <c r="L40" s="186"/>
+      <c r="M40" s="186"/>
+      <c r="N40" s="186"/>
+      <c r="O40" s="186"/>
+      <c r="P40" s="186"/>
+      <c r="Q40" s="186"/>
+      <c r="R40" s="186"/>
+      <c r="S40" s="186"/>
+      <c r="T40" s="186"/>
+      <c r="U40" s="186"/>
+      <c r="V40" s="186"/>
+      <c r="W40" s="201" t="s">
+        <v>13</v>
+      </c>
+      <c r="X40" s="201"/>
+      <c r="Y40" s="202"/>
+      <c r="Z40" s="202"/>
+      <c r="AA40" s="203"/>
+      <c r="AB40" s="203"/>
+      <c r="AC40" s="203"/>
+      <c r="AD40" s="203"/>
+      <c r="AE40" s="203"/>
+      <c r="AF40" s="203"/>
+      <c r="AG40" s="202"/>
+      <c r="AH40" s="203"/>
       <c r="AI40" s="42"/>
       <c r="AJ40" s="85"/>
       <c r="AK40" s="85"/>
@@ -4325,34 +4384,34 @@
     </row>
     <row r="41" spans="1:45" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="16"/>
-      <c r="B41" s="99" t="s">
+      <c r="B41" s="136" t="s">
         <v>35</v>
       </c>
-      <c r="C41" s="99"/>
-      <c r="D41" s="99"/>
-      <c r="E41" s="99"/>
-      <c r="F41" s="99"/>
-      <c r="G41" s="99"/>
-      <c r="H41" s="99"/>
-      <c r="I41" s="99"/>
-      <c r="J41" s="99"/>
-      <c r="K41" s="99"/>
-      <c r="L41" s="99"/>
-      <c r="M41" s="99"/>
-      <c r="N41" s="99"/>
-      <c r="O41" s="99"/>
-      <c r="P41" s="99"/>
-      <c r="Q41" s="99"/>
-      <c r="R41" s="99"/>
-      <c r="S41" s="99"/>
-      <c r="T41" s="99"/>
-      <c r="U41" s="99"/>
-      <c r="V41" s="99"/>
-      <c r="W41" s="99"/>
-      <c r="X41" s="99"/>
-      <c r="Y41" s="99"/>
-      <c r="Z41" s="99"/>
-      <c r="AA41" s="99"/>
+      <c r="C41" s="136"/>
+      <c r="D41" s="136"/>
+      <c r="E41" s="136"/>
+      <c r="F41" s="136"/>
+      <c r="G41" s="136"/>
+      <c r="H41" s="136"/>
+      <c r="I41" s="136"/>
+      <c r="J41" s="136"/>
+      <c r="K41" s="136"/>
+      <c r="L41" s="136"/>
+      <c r="M41" s="136"/>
+      <c r="N41" s="136"/>
+      <c r="O41" s="136"/>
+      <c r="P41" s="136"/>
+      <c r="Q41" s="136"/>
+      <c r="R41" s="136"/>
+      <c r="S41" s="136"/>
+      <c r="T41" s="136"/>
+      <c r="U41" s="136"/>
+      <c r="V41" s="136"/>
+      <c r="W41" s="136"/>
+      <c r="X41" s="136"/>
+      <c r="Y41" s="136"/>
+      <c r="Z41" s="136"/>
+      <c r="AA41" s="136"/>
       <c r="AB41" s="43"/>
       <c r="AC41" s="43"/>
       <c r="AD41" s="43"/>
@@ -4407,18 +4466,18 @@
       <c r="T42" s="80"/>
       <c r="U42" s="79"/>
       <c r="V42" s="80"/>
-      <c r="W42" s="96"/>
-      <c r="X42" s="103"/>
-      <c r="Y42" s="103"/>
-      <c r="Z42" s="103"/>
-      <c r="AA42" s="103"/>
-      <c r="AB42" s="103"/>
-      <c r="AC42" s="103"/>
-      <c r="AD42" s="103"/>
-      <c r="AE42" s="103"/>
-      <c r="AF42" s="103"/>
-      <c r="AG42" s="103"/>
-      <c r="AH42" s="97"/>
+      <c r="W42" s="106"/>
+      <c r="X42" s="117"/>
+      <c r="Y42" s="117"/>
+      <c r="Z42" s="117"/>
+      <c r="AA42" s="117"/>
+      <c r="AB42" s="117"/>
+      <c r="AC42" s="117"/>
+      <c r="AD42" s="117"/>
+      <c r="AE42" s="117"/>
+      <c r="AF42" s="117"/>
+      <c r="AG42" s="117"/>
+      <c r="AH42" s="107"/>
       <c r="AI42" s="49"/>
       <c r="AJ42" s="85"/>
       <c r="AK42" s="85"/>
@@ -4434,39 +4493,39 @@
     <row r="43" spans="1:45" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="45"/>
       <c r="F43" s="50"/>
-      <c r="G43" s="108" t="s">
+      <c r="G43" s="193" t="s">
         <v>6</v>
       </c>
-      <c r="H43" s="108"/>
-      <c r="I43" s="108"/>
-      <c r="K43" s="109" t="s">
+      <c r="H43" s="193"/>
+      <c r="I43" s="193"/>
+      <c r="K43" s="121" t="s">
         <v>7</v>
       </c>
-      <c r="L43" s="109"/>
-      <c r="M43" s="109"/>
-      <c r="N43" s="109"/>
-      <c r="O43" s="109"/>
-      <c r="P43" s="109"/>
-      <c r="Q43" s="109"/>
-      <c r="R43" s="109"/>
-      <c r="S43" s="109"/>
+      <c r="L43" s="121"/>
+      <c r="M43" s="121"/>
+      <c r="N43" s="121"/>
+      <c r="O43" s="121"/>
+      <c r="P43" s="121"/>
+      <c r="Q43" s="121"/>
+      <c r="R43" s="121"/>
+      <c r="S43" s="121"/>
       <c r="T43" s="43"/>
       <c r="U43" s="51"/>
       <c r="V43" s="43"/>
-      <c r="W43" s="131" t="s">
+      <c r="W43" s="154" t="s">
         <v>34</v>
       </c>
-      <c r="X43" s="131"/>
-      <c r="Y43" s="131"/>
-      <c r="Z43" s="131"/>
-      <c r="AA43" s="131"/>
-      <c r="AB43" s="131"/>
-      <c r="AC43" s="131"/>
-      <c r="AD43" s="131"/>
-      <c r="AE43" s="131"/>
-      <c r="AF43" s="131"/>
-      <c r="AG43" s="131"/>
-      <c r="AH43" s="131"/>
+      <c r="X43" s="154"/>
+      <c r="Y43" s="154"/>
+      <c r="Z43" s="154"/>
+      <c r="AA43" s="154"/>
+      <c r="AB43" s="154"/>
+      <c r="AC43" s="154"/>
+      <c r="AD43" s="154"/>
+      <c r="AE43" s="154"/>
+      <c r="AF43" s="154"/>
+      <c r="AG43" s="154"/>
+      <c r="AH43" s="154"/>
       <c r="AI43" s="49"/>
       <c r="AJ43" s="85"/>
       <c r="AK43" s="85"/>
@@ -4480,45 +4539,45 @@
       <c r="AS43" s="85"/>
     </row>
     <row r="44" spans="1:45" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="133" t="s">
+      <c r="A44" s="189" t="s">
         <v>82</v>
       </c>
-      <c r="B44" s="133"/>
-      <c r="C44" s="133"/>
-      <c r="D44" s="133"/>
-      <c r="E44" s="133" t="s">
+      <c r="B44" s="189"/>
+      <c r="C44" s="189"/>
+      <c r="D44" s="189"/>
+      <c r="E44" s="189" t="s">
         <v>83</v>
       </c>
-      <c r="F44" s="133"/>
-      <c r="G44" s="133"/>
-      <c r="H44" s="133"/>
-      <c r="I44" s="133"/>
-      <c r="J44" s="133"/>
-      <c r="K44" s="133"/>
-      <c r="L44" s="133"/>
-      <c r="M44" s="133"/>
-      <c r="N44" s="133"/>
-      <c r="O44" s="133"/>
-      <c r="P44" s="133"/>
-      <c r="Q44" s="133"/>
-      <c r="R44" s="133"/>
-      <c r="S44" s="133"/>
-      <c r="T44" s="133"/>
-      <c r="U44" s="133"/>
-      <c r="V44" s="133"/>
-      <c r="W44" s="133"/>
-      <c r="X44" s="133"/>
-      <c r="Y44" s="133"/>
-      <c r="Z44" s="133"/>
-      <c r="AA44" s="133"/>
-      <c r="AB44" s="133"/>
-      <c r="AC44" s="133"/>
-      <c r="AD44" s="133"/>
-      <c r="AE44" s="133"/>
-      <c r="AF44" s="133"/>
-      <c r="AG44" s="133"/>
-      <c r="AH44" s="133"/>
-      <c r="AI44" s="133"/>
+      <c r="F44" s="189"/>
+      <c r="G44" s="189"/>
+      <c r="H44" s="189"/>
+      <c r="I44" s="189"/>
+      <c r="J44" s="189"/>
+      <c r="K44" s="189"/>
+      <c r="L44" s="189"/>
+      <c r="M44" s="189"/>
+      <c r="N44" s="189"/>
+      <c r="O44" s="189"/>
+      <c r="P44" s="189"/>
+      <c r="Q44" s="189"/>
+      <c r="R44" s="189"/>
+      <c r="S44" s="189"/>
+      <c r="T44" s="189"/>
+      <c r="U44" s="189"/>
+      <c r="V44" s="189"/>
+      <c r="W44" s="189"/>
+      <c r="X44" s="189"/>
+      <c r="Y44" s="189"/>
+      <c r="Z44" s="189"/>
+      <c r="AA44" s="189"/>
+      <c r="AB44" s="189"/>
+      <c r="AC44" s="189"/>
+      <c r="AD44" s="189"/>
+      <c r="AE44" s="189"/>
+      <c r="AF44" s="189"/>
+      <c r="AG44" s="189"/>
+      <c r="AH44" s="189"/>
+      <c r="AI44" s="189"/>
       <c r="AJ44" s="91"/>
       <c r="AK44" s="85"/>
       <c r="AL44" s="85"/>
@@ -4531,43 +4590,43 @@
       <c r="AS44" s="85"/>
     </row>
     <row r="45" spans="1:45" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="133"/>
-      <c r="B45" s="133"/>
-      <c r="C45" s="133"/>
-      <c r="D45" s="133"/>
-      <c r="E45" s="133" t="s">
+      <c r="A45" s="189"/>
+      <c r="B45" s="189"/>
+      <c r="C45" s="189"/>
+      <c r="D45" s="189"/>
+      <c r="E45" s="189" t="s">
         <v>86</v>
       </c>
-      <c r="F45" s="133"/>
-      <c r="G45" s="133"/>
-      <c r="H45" s="133"/>
-      <c r="I45" s="133"/>
-      <c r="J45" s="133"/>
-      <c r="K45" s="133"/>
-      <c r="L45" s="133"/>
-      <c r="M45" s="133"/>
-      <c r="N45" s="133"/>
-      <c r="O45" s="133"/>
-      <c r="P45" s="133"/>
-      <c r="Q45" s="133"/>
-      <c r="R45" s="133"/>
-      <c r="S45" s="133"/>
-      <c r="T45" s="133"/>
-      <c r="U45" s="133"/>
-      <c r="V45" s="133"/>
-      <c r="W45" s="133"/>
-      <c r="X45" s="133"/>
-      <c r="Y45" s="133"/>
-      <c r="Z45" s="133"/>
-      <c r="AA45" s="133"/>
-      <c r="AB45" s="133"/>
-      <c r="AC45" s="133"/>
-      <c r="AD45" s="133"/>
-      <c r="AE45" s="133"/>
-      <c r="AF45" s="133"/>
-      <c r="AG45" s="133"/>
-      <c r="AH45" s="133"/>
-      <c r="AI45" s="133"/>
+      <c r="F45" s="189"/>
+      <c r="G45" s="189"/>
+      <c r="H45" s="189"/>
+      <c r="I45" s="189"/>
+      <c r="J45" s="189"/>
+      <c r="K45" s="189"/>
+      <c r="L45" s="189"/>
+      <c r="M45" s="189"/>
+      <c r="N45" s="189"/>
+      <c r="O45" s="189"/>
+      <c r="P45" s="189"/>
+      <c r="Q45" s="189"/>
+      <c r="R45" s="189"/>
+      <c r="S45" s="189"/>
+      <c r="T45" s="189"/>
+      <c r="U45" s="189"/>
+      <c r="V45" s="189"/>
+      <c r="W45" s="189"/>
+      <c r="X45" s="189"/>
+      <c r="Y45" s="189"/>
+      <c r="Z45" s="189"/>
+      <c r="AA45" s="189"/>
+      <c r="AB45" s="189"/>
+      <c r="AC45" s="189"/>
+      <c r="AD45" s="189"/>
+      <c r="AE45" s="189"/>
+      <c r="AF45" s="189"/>
+      <c r="AG45" s="189"/>
+      <c r="AH45" s="189"/>
+      <c r="AI45" s="189"/>
       <c r="AJ45" s="83"/>
     </row>
     <row r="46" spans="1:45" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4575,37 +4634,37 @@
       <c r="B46" s="52"/>
       <c r="C46" s="52"/>
       <c r="D46" s="52"/>
-      <c r="E46" s="134" t="s">
+      <c r="E46" s="190" t="s">
         <v>81</v>
       </c>
-      <c r="F46" s="134"/>
-      <c r="G46" s="134"/>
-      <c r="H46" s="134"/>
-      <c r="I46" s="134"/>
-      <c r="J46" s="134"/>
-      <c r="K46" s="134"/>
-      <c r="L46" s="134"/>
-      <c r="M46" s="100"/>
-      <c r="N46" s="101"/>
-      <c r="O46" s="101"/>
-      <c r="P46" s="101"/>
-      <c r="Q46" s="101"/>
-      <c r="R46" s="101"/>
-      <c r="S46" s="101"/>
-      <c r="T46" s="101"/>
-      <c r="U46" s="102"/>
-      <c r="V46" s="135" t="s">
+      <c r="F46" s="190"/>
+      <c r="G46" s="190"/>
+      <c r="H46" s="190"/>
+      <c r="I46" s="190"/>
+      <c r="J46" s="190"/>
+      <c r="K46" s="190"/>
+      <c r="L46" s="190"/>
+      <c r="M46" s="114"/>
+      <c r="N46" s="115"/>
+      <c r="O46" s="115"/>
+      <c r="P46" s="115"/>
+      <c r="Q46" s="115"/>
+      <c r="R46" s="115"/>
+      <c r="S46" s="115"/>
+      <c r="T46" s="115"/>
+      <c r="U46" s="116"/>
+      <c r="V46" s="191" t="s">
         <v>21</v>
       </c>
-      <c r="W46" s="136"/>
-      <c r="X46" s="96"/>
-      <c r="Y46" s="97"/>
-      <c r="Z46" s="96"/>
-      <c r="AA46" s="97"/>
-      <c r="AB46" s="96" t="s">
+      <c r="W46" s="192"/>
+      <c r="X46" s="106"/>
+      <c r="Y46" s="107"/>
+      <c r="Z46" s="106"/>
+      <c r="AA46" s="107"/>
+      <c r="AB46" s="106" t="s">
         <v>118</v>
       </c>
-      <c r="AC46" s="97"/>
+      <c r="AC46" s="107"/>
       <c r="AD46" s="52"/>
       <c r="AE46" s="52"/>
       <c r="AF46" s="52"/>
@@ -4624,34 +4683,34 @@
       <c r="G47" s="52"/>
       <c r="H47" s="52"/>
       <c r="I47" s="52"/>
-      <c r="J47" s="132" t="s">
+      <c r="J47" s="188" t="s">
         <v>84</v>
       </c>
-      <c r="K47" s="132"/>
-      <c r="L47" s="132"/>
-      <c r="M47" s="132"/>
-      <c r="N47" s="132"/>
-      <c r="O47" s="132"/>
-      <c r="P47" s="132"/>
-      <c r="Q47" s="132"/>
-      <c r="R47" s="132"/>
-      <c r="S47" s="132"/>
-      <c r="T47" s="132"/>
-      <c r="U47" s="132"/>
-      <c r="V47" s="132"/>
-      <c r="W47" s="132"/>
-      <c r="X47" s="115" t="s">
+      <c r="K47" s="188"/>
+      <c r="L47" s="188"/>
+      <c r="M47" s="188"/>
+      <c r="N47" s="188"/>
+      <c r="O47" s="188"/>
+      <c r="P47" s="188"/>
+      <c r="Q47" s="188"/>
+      <c r="R47" s="188"/>
+      <c r="S47" s="188"/>
+      <c r="T47" s="188"/>
+      <c r="U47" s="188"/>
+      <c r="V47" s="188"/>
+      <c r="W47" s="188"/>
+      <c r="X47" s="155" t="s">
         <v>24</v>
       </c>
-      <c r="Y47" s="115"/>
-      <c r="Z47" s="115" t="s">
+      <c r="Y47" s="155"/>
+      <c r="Z47" s="155" t="s">
         <v>25</v>
       </c>
-      <c r="AA47" s="115"/>
-      <c r="AB47" s="115" t="s">
+      <c r="AA47" s="155"/>
+      <c r="AB47" s="155" t="s">
         <v>26</v>
       </c>
-      <c r="AC47" s="115"/>
+      <c r="AC47" s="155"/>
       <c r="AD47" s="52"/>
       <c r="AE47" s="52"/>
       <c r="AF47" s="52"/>
@@ -4698,109 +4757,109 @@
       <c r="AI48" s="28"/>
     </row>
     <row r="49" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="B49" s="116"/>
-      <c r="C49" s="117"/>
-      <c r="D49" s="117"/>
-      <c r="E49" s="117"/>
-      <c r="F49" s="117"/>
-      <c r="G49" s="117"/>
-      <c r="H49" s="117"/>
-      <c r="I49" s="117"/>
-      <c r="J49" s="117"/>
-      <c r="K49" s="117"/>
-      <c r="L49" s="117"/>
-      <c r="M49" s="117"/>
-      <c r="N49" s="117"/>
-      <c r="O49" s="118"/>
-      <c r="Q49" s="122"/>
-      <c r="R49" s="123"/>
-      <c r="S49" s="123"/>
-      <c r="T49" s="123"/>
-      <c r="U49" s="123"/>
-      <c r="V49" s="123"/>
-      <c r="W49" s="123"/>
-      <c r="X49" s="124"/>
-      <c r="Z49" s="116"/>
-      <c r="AA49" s="117"/>
-      <c r="AB49" s="117"/>
-      <c r="AC49" s="117"/>
-      <c r="AD49" s="117"/>
-      <c r="AE49" s="117"/>
-      <c r="AF49" s="117"/>
-      <c r="AG49" s="117"/>
-      <c r="AH49" s="118"/>
+      <c r="B49" s="171"/>
+      <c r="C49" s="172"/>
+      <c r="D49" s="172"/>
+      <c r="E49" s="172"/>
+      <c r="F49" s="172"/>
+      <c r="G49" s="172"/>
+      <c r="H49" s="172"/>
+      <c r="I49" s="172"/>
+      <c r="J49" s="172"/>
+      <c r="K49" s="172"/>
+      <c r="L49" s="172"/>
+      <c r="M49" s="172"/>
+      <c r="N49" s="172"/>
+      <c r="O49" s="173"/>
+      <c r="Q49" s="177"/>
+      <c r="R49" s="178"/>
+      <c r="S49" s="178"/>
+      <c r="T49" s="178"/>
+      <c r="U49" s="178"/>
+      <c r="V49" s="178"/>
+      <c r="W49" s="178"/>
+      <c r="X49" s="179"/>
+      <c r="Z49" s="171"/>
+      <c r="AA49" s="172"/>
+      <c r="AB49" s="172"/>
+      <c r="AC49" s="172"/>
+      <c r="AD49" s="172"/>
+      <c r="AE49" s="172"/>
+      <c r="AF49" s="172"/>
+      <c r="AG49" s="172"/>
+      <c r="AH49" s="173"/>
       <c r="AI49" s="53"/>
     </row>
     <row r="50" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="B50" s="119"/>
-      <c r="C50" s="120"/>
-      <c r="D50" s="120"/>
-      <c r="E50" s="120"/>
-      <c r="F50" s="120"/>
-      <c r="G50" s="120"/>
-      <c r="H50" s="120"/>
-      <c r="I50" s="120"/>
-      <c r="J50" s="120"/>
-      <c r="K50" s="120"/>
-      <c r="L50" s="120"/>
-      <c r="M50" s="120"/>
-      <c r="N50" s="120"/>
-      <c r="O50" s="121"/>
-      <c r="Q50" s="125"/>
-      <c r="R50" s="126"/>
-      <c r="S50" s="126"/>
-      <c r="T50" s="126"/>
-      <c r="U50" s="126"/>
-      <c r="V50" s="126"/>
-      <c r="W50" s="126"/>
-      <c r="X50" s="127"/>
-      <c r="Z50" s="119"/>
-      <c r="AA50" s="120"/>
-      <c r="AB50" s="120"/>
-      <c r="AC50" s="120"/>
-      <c r="AD50" s="120"/>
-      <c r="AE50" s="120"/>
-      <c r="AF50" s="120"/>
-      <c r="AG50" s="120"/>
-      <c r="AH50" s="121"/>
+      <c r="B50" s="174"/>
+      <c r="C50" s="175"/>
+      <c r="D50" s="175"/>
+      <c r="E50" s="175"/>
+      <c r="F50" s="175"/>
+      <c r="G50" s="175"/>
+      <c r="H50" s="175"/>
+      <c r="I50" s="175"/>
+      <c r="J50" s="175"/>
+      <c r="K50" s="175"/>
+      <c r="L50" s="175"/>
+      <c r="M50" s="175"/>
+      <c r="N50" s="175"/>
+      <c r="O50" s="176"/>
+      <c r="Q50" s="180"/>
+      <c r="R50" s="181"/>
+      <c r="S50" s="181"/>
+      <c r="T50" s="181"/>
+      <c r="U50" s="181"/>
+      <c r="V50" s="181"/>
+      <c r="W50" s="181"/>
+      <c r="X50" s="182"/>
+      <c r="Z50" s="174"/>
+      <c r="AA50" s="175"/>
+      <c r="AB50" s="175"/>
+      <c r="AC50" s="175"/>
+      <c r="AD50" s="175"/>
+      <c r="AE50" s="175"/>
+      <c r="AF50" s="175"/>
+      <c r="AG50" s="175"/>
+      <c r="AH50" s="176"/>
       <c r="AI50" s="53"/>
     </row>
     <row r="51" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="B51" s="110" t="s">
+      <c r="B51" s="186" t="s">
         <v>80</v>
       </c>
-      <c r="C51" s="110"/>
-      <c r="D51" s="110"/>
-      <c r="E51" s="110"/>
-      <c r="F51" s="110"/>
-      <c r="G51" s="110"/>
-      <c r="H51" s="110"/>
-      <c r="I51" s="110"/>
-      <c r="J51" s="110"/>
-      <c r="K51" s="110"/>
-      <c r="L51" s="110"/>
-      <c r="M51" s="110"/>
-      <c r="N51" s="110"/>
-      <c r="O51" s="110"/>
-      <c r="Q51" s="128"/>
-      <c r="R51" s="129"/>
-      <c r="S51" s="129"/>
-      <c r="T51" s="129"/>
-      <c r="U51" s="129"/>
-      <c r="V51" s="129"/>
-      <c r="W51" s="129"/>
-      <c r="X51" s="130"/>
-      <c r="Z51" s="108" t="s">
+      <c r="C51" s="186"/>
+      <c r="D51" s="186"/>
+      <c r="E51" s="186"/>
+      <c r="F51" s="186"/>
+      <c r="G51" s="186"/>
+      <c r="H51" s="186"/>
+      <c r="I51" s="186"/>
+      <c r="J51" s="186"/>
+      <c r="K51" s="186"/>
+      <c r="L51" s="186"/>
+      <c r="M51" s="186"/>
+      <c r="N51" s="186"/>
+      <c r="O51" s="186"/>
+      <c r="Q51" s="183"/>
+      <c r="R51" s="184"/>
+      <c r="S51" s="184"/>
+      <c r="T51" s="184"/>
+      <c r="U51" s="184"/>
+      <c r="V51" s="184"/>
+      <c r="W51" s="184"/>
+      <c r="X51" s="185"/>
+      <c r="Z51" s="193" t="s">
         <v>0</v>
       </c>
-      <c r="AA51" s="108"/>
-      <c r="AB51" s="108"/>
-      <c r="AC51" s="108"/>
-      <c r="AD51" s="108"/>
-      <c r="AE51" s="108"/>
-      <c r="AF51" s="108"/>
-      <c r="AG51" s="108"/>
-      <c r="AH51" s="108"/>
+      <c r="AA51" s="193"/>
+      <c r="AB51" s="193"/>
+      <c r="AC51" s="193"/>
+      <c r="AD51" s="193"/>
+      <c r="AE51" s="193"/>
+      <c r="AF51" s="193"/>
+      <c r="AG51" s="193"/>
+      <c r="AH51" s="193"/>
       <c r="AI51" s="4"/>
     </row>
     <row r="52" spans="1:35" ht="12" customHeight="1" x14ac:dyDescent="0.25">
@@ -4808,16 +4867,16 @@
         <v>8</v>
       </c>
       <c r="O52" s="54"/>
-      <c r="Q52" s="114" t="s">
+      <c r="Q52" s="170" t="s">
         <v>1</v>
       </c>
-      <c r="R52" s="114"/>
-      <c r="S52" s="114"/>
-      <c r="T52" s="114"/>
-      <c r="U52" s="114"/>
-      <c r="V52" s="114"/>
-      <c r="W52" s="114"/>
-      <c r="X52" s="114"/>
+      <c r="R52" s="170"/>
+      <c r="S52" s="170"/>
+      <c r="T52" s="170"/>
+      <c r="U52" s="170"/>
+      <c r="V52" s="170"/>
+      <c r="W52" s="170"/>
+      <c r="X52" s="170"/>
     </row>
     <row r="53" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B53" s="55" t="s">
@@ -4838,27 +4897,27 @@
       <c r="O53" s="55"/>
       <c r="P53" s="55"/>
       <c r="Q53" s="55"/>
-      <c r="R53" s="96"/>
-      <c r="S53" s="103"/>
-      <c r="T53" s="103"/>
-      <c r="U53" s="97"/>
+      <c r="R53" s="106"/>
+      <c r="S53" s="117"/>
+      <c r="T53" s="117"/>
+      <c r="U53" s="107"/>
       <c r="V53" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="W53" s="96"/>
-      <c r="X53" s="97"/>
-      <c r="Y53" s="96"/>
-      <c r="Z53" s="97"/>
-      <c r="AA53" s="96"/>
-      <c r="AB53" s="97"/>
+      <c r="W53" s="106"/>
+      <c r="X53" s="107"/>
+      <c r="Y53" s="106"/>
+      <c r="Z53" s="107"/>
+      <c r="AA53" s="106"/>
+      <c r="AB53" s="107"/>
       <c r="AC53" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="AD53" s="96"/>
-      <c r="AE53" s="103"/>
-      <c r="AF53" s="103"/>
-      <c r="AG53" s="103"/>
-      <c r="AH53" s="97"/>
+      <c r="AD53" s="106"/>
+      <c r="AE53" s="117"/>
+      <c r="AF53" s="117"/>
+      <c r="AG53" s="117"/>
+      <c r="AH53" s="107"/>
     </row>
     <row r="54" spans="1:35" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="55"/>
@@ -4896,73 +4955,73 @@
       <c r="AH54" s="92"/>
     </row>
     <row r="55" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="161" t="s">
+      <c r="B55" s="163" t="s">
         <v>37</v>
       </c>
-      <c r="C55" s="162"/>
-      <c r="D55" s="162"/>
-      <c r="E55" s="162"/>
-      <c r="F55" s="162"/>
-      <c r="G55" s="162"/>
-      <c r="H55" s="162"/>
-      <c r="I55" s="162"/>
-      <c r="J55" s="162"/>
-      <c r="K55" s="162"/>
-      <c r="L55" s="162"/>
-      <c r="M55" s="162"/>
-      <c r="N55" s="162"/>
-      <c r="O55" s="162"/>
+      <c r="C55" s="164"/>
+      <c r="D55" s="164"/>
+      <c r="E55" s="164"/>
+      <c r="F55" s="164"/>
+      <c r="G55" s="164"/>
+      <c r="H55" s="164"/>
+      <c r="I55" s="164"/>
+      <c r="J55" s="164"/>
+      <c r="K55" s="164"/>
+      <c r="L55" s="164"/>
+      <c r="M55" s="164"/>
+      <c r="N55" s="164"/>
+      <c r="O55" s="164"/>
       <c r="P55" s="57"/>
       <c r="Q55" s="57"/>
-      <c r="R55" s="115" t="s">
+      <c r="R55" s="155" t="s">
         <v>23</v>
       </c>
-      <c r="S55" s="115"/>
-      <c r="T55" s="115"/>
-      <c r="U55" s="115"/>
+      <c r="S55" s="155"/>
+      <c r="T55" s="155"/>
+      <c r="U55" s="155"/>
       <c r="V55" s="57"/>
-      <c r="W55" s="115" t="s">
+      <c r="W55" s="155" t="s">
         <v>24</v>
       </c>
-      <c r="X55" s="115"/>
-      <c r="Y55" s="115" t="s">
+      <c r="X55" s="155"/>
+      <c r="Y55" s="155" t="s">
         <v>25</v>
       </c>
-      <c r="Z55" s="115"/>
-      <c r="AA55" s="115" t="s">
+      <c r="Z55" s="155"/>
+      <c r="AA55" s="155" t="s">
         <v>26</v>
       </c>
-      <c r="AB55" s="115"/>
+      <c r="AB55" s="155"/>
       <c r="AC55" s="57"/>
-      <c r="AD55" s="115" t="s">
+      <c r="AD55" s="155" t="s">
         <v>27</v>
       </c>
-      <c r="AE55" s="115"/>
-      <c r="AF55" s="115"/>
-      <c r="AG55" s="115"/>
-      <c r="AH55" s="115"/>
+      <c r="AE55" s="155"/>
+      <c r="AF55" s="155"/>
+      <c r="AG55" s="155"/>
+      <c r="AH55" s="155"/>
     </row>
     <row r="56" spans="1:35" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="158"/>
-      <c r="C56" s="158"/>
-      <c r="D56" s="158"/>
-      <c r="E56" s="158"/>
-      <c r="F56" s="158"/>
-      <c r="G56" s="158"/>
-      <c r="H56" s="158"/>
-      <c r="I56" s="158"/>
-      <c r="J56" s="158"/>
-      <c r="K56" s="158"/>
-      <c r="L56" s="158"/>
-      <c r="M56" s="158"/>
-      <c r="N56" s="158"/>
-      <c r="O56" s="158"/>
-      <c r="P56" s="158"/>
+      <c r="B56" s="160"/>
+      <c r="C56" s="160"/>
+      <c r="D56" s="160"/>
+      <c r="E56" s="160"/>
+      <c r="F56" s="160"/>
+      <c r="G56" s="160"/>
+      <c r="H56" s="160"/>
+      <c r="I56" s="160"/>
+      <c r="J56" s="160"/>
+      <c r="K56" s="160"/>
+      <c r="L56" s="160"/>
+      <c r="M56" s="160"/>
+      <c r="N56" s="160"/>
+      <c r="O56" s="160"/>
+      <c r="P56" s="160"/>
       <c r="Q56" s="58"/>
-      <c r="R56" s="154"/>
-      <c r="S56" s="154"/>
-      <c r="T56" s="154"/>
-      <c r="U56" s="154"/>
+      <c r="R56" s="156"/>
+      <c r="S56" s="156"/>
+      <c r="T56" s="156"/>
+      <c r="U56" s="156"/>
       <c r="V56" s="57"/>
       <c r="W56" s="57"/>
       <c r="X56" s="50"/>
@@ -4971,18 +5030,18 @@
       <c r="AA56" s="50"/>
       <c r="AB56" s="50"/>
       <c r="AC56" s="59"/>
-      <c r="AD56" s="155"/>
-      <c r="AE56" s="155"/>
-      <c r="AF56" s="155"/>
-      <c r="AG56" s="155"/>
-      <c r="AH56" s="155"/>
+      <c r="AD56" s="157"/>
+      <c r="AE56" s="157"/>
+      <c r="AF56" s="157"/>
+      <c r="AG56" s="157"/>
+      <c r="AH56" s="157"/>
     </row>
     <row r="57" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A57" s="60"/>
-      <c r="B57" s="138" t="s">
+      <c r="B57" s="108" t="s">
         <v>2</v>
       </c>
-      <c r="C57" s="138"/>
+      <c r="C57" s="108"/>
       <c r="D57" s="139"/>
       <c r="E57" s="61">
         <v>8</v>
@@ -5034,17 +5093,17 @@
       </c>
       <c r="H58" s="149"/>
       <c r="I58" s="149"/>
-      <c r="K58" s="109" t="s">
+      <c r="K58" s="121" t="s">
         <v>7</v>
       </c>
-      <c r="L58" s="109"/>
-      <c r="M58" s="109"/>
-      <c r="N58" s="109"/>
-      <c r="O58" s="109"/>
-      <c r="P58" s="109"/>
-      <c r="Q58" s="109"/>
-      <c r="R58" s="109"/>
-      <c r="S58" s="109"/>
+      <c r="L58" s="121"/>
+      <c r="M58" s="121"/>
+      <c r="N58" s="121"/>
+      <c r="O58" s="121"/>
+      <c r="P58" s="121"/>
+      <c r="Q58" s="121"/>
+      <c r="R58" s="121"/>
+      <c r="S58" s="121"/>
       <c r="T58" s="49"/>
       <c r="V58" s="143"/>
       <c r="W58" s="144"/>
@@ -5102,17 +5161,17 @@
       <c r="B60" s="153" t="s">
         <v>38</v>
       </c>
-      <c r="C60" s="131"/>
-      <c r="D60" s="131"/>
-      <c r="E60" s="131"/>
-      <c r="F60" s="131"/>
-      <c r="G60" s="131"/>
-      <c r="H60" s="131"/>
-      <c r="I60" s="131"/>
-      <c r="J60" s="131"/>
-      <c r="K60" s="131"/>
-      <c r="L60" s="131"/>
-      <c r="M60" s="131"/>
+      <c r="C60" s="154"/>
+      <c r="D60" s="154"/>
+      <c r="E60" s="154"/>
+      <c r="F60" s="154"/>
+      <c r="G60" s="154"/>
+      <c r="H60" s="154"/>
+      <c r="I60" s="154"/>
+      <c r="J60" s="154"/>
+      <c r="K60" s="154"/>
+      <c r="L60" s="154"/>
+      <c r="M60" s="154"/>
       <c r="N60" s="49"/>
       <c r="O60" s="49"/>
       <c r="P60" s="49"/>
@@ -5137,18 +5196,18 @@
     </row>
     <row r="61" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="14"/>
-      <c r="B61" s="163"/>
-      <c r="C61" s="164"/>
-      <c r="D61" s="164"/>
-      <c r="E61" s="164"/>
-      <c r="F61" s="164"/>
-      <c r="G61" s="164"/>
-      <c r="H61" s="164"/>
-      <c r="I61" s="164"/>
-      <c r="J61" s="164"/>
-      <c r="K61" s="164"/>
-      <c r="L61" s="164"/>
-      <c r="M61" s="165"/>
+      <c r="B61" s="165"/>
+      <c r="C61" s="166"/>
+      <c r="D61" s="166"/>
+      <c r="E61" s="166"/>
+      <c r="F61" s="166"/>
+      <c r="G61" s="166"/>
+      <c r="H61" s="166"/>
+      <c r="I61" s="166"/>
+      <c r="J61" s="166"/>
+      <c r="K61" s="166"/>
+      <c r="L61" s="166"/>
+      <c r="M61" s="167"/>
       <c r="N61" s="49"/>
       <c r="O61" s="49"/>
       <c r="P61" s="49"/>
@@ -5173,20 +5232,20 @@
     </row>
     <row r="62" spans="1:35" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="14"/>
-      <c r="B62" s="166" t="s">
+      <c r="B62" s="168" t="s">
         <v>117</v>
       </c>
-      <c r="C62" s="167"/>
-      <c r="D62" s="167"/>
-      <c r="E62" s="167"/>
-      <c r="F62" s="167"/>
-      <c r="G62" s="167"/>
-      <c r="H62" s="167"/>
-      <c r="I62" s="167"/>
-      <c r="J62" s="167"/>
-      <c r="K62" s="167"/>
-      <c r="L62" s="167"/>
-      <c r="M62" s="167"/>
+      <c r="C62" s="169"/>
+      <c r="D62" s="169"/>
+      <c r="E62" s="169"/>
+      <c r="F62" s="169"/>
+      <c r="G62" s="169"/>
+      <c r="H62" s="169"/>
+      <c r="I62" s="169"/>
+      <c r="J62" s="169"/>
+      <c r="K62" s="169"/>
+      <c r="L62" s="169"/>
+      <c r="M62" s="169"/>
       <c r="N62" s="49"/>
       <c r="O62" s="49"/>
       <c r="P62" s="49"/>
@@ -5210,313 +5269,339 @@
       <c r="AI62" s="93"/>
     </row>
     <row r="63" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="159" t="s">
+      <c r="A63" s="161" t="s">
         <v>85</v>
       </c>
-      <c r="B63" s="159"/>
-      <c r="C63" s="159"/>
-      <c r="D63" s="159"/>
-      <c r="E63" s="159"/>
-      <c r="F63" s="159"/>
-      <c r="G63" s="159"/>
-      <c r="H63" s="159"/>
-      <c r="I63" s="159"/>
-      <c r="J63" s="159"/>
-      <c r="K63" s="159"/>
-      <c r="L63" s="159"/>
-      <c r="M63" s="159"/>
-      <c r="N63" s="159"/>
-      <c r="O63" s="159"/>
-      <c r="P63" s="159"/>
-      <c r="Q63" s="159"/>
-      <c r="R63" s="159"/>
-      <c r="S63" s="159"/>
-      <c r="T63" s="159"/>
-      <c r="U63" s="159"/>
-      <c r="V63" s="159"/>
-      <c r="W63" s="159"/>
-      <c r="X63" s="159"/>
-      <c r="Y63" s="159"/>
-      <c r="Z63" s="159"/>
-      <c r="AA63" s="159"/>
-      <c r="AB63" s="159"/>
-      <c r="AC63" s="159"/>
-      <c r="AD63" s="159"/>
-      <c r="AE63" s="159"/>
-      <c r="AF63" s="159"/>
-      <c r="AG63" s="159"/>
-      <c r="AH63" s="159"/>
-      <c r="AI63" s="159"/>
+      <c r="B63" s="161"/>
+      <c r="C63" s="161"/>
+      <c r="D63" s="161"/>
+      <c r="E63" s="161"/>
+      <c r="F63" s="161"/>
+      <c r="G63" s="161"/>
+      <c r="H63" s="161"/>
+      <c r="I63" s="161"/>
+      <c r="J63" s="161"/>
+      <c r="K63" s="161"/>
+      <c r="L63" s="161"/>
+      <c r="M63" s="161"/>
+      <c r="N63" s="161"/>
+      <c r="O63" s="161"/>
+      <c r="P63" s="161"/>
+      <c r="Q63" s="161"/>
+      <c r="R63" s="161"/>
+      <c r="S63" s="161"/>
+      <c r="T63" s="161"/>
+      <c r="U63" s="161"/>
+      <c r="V63" s="161"/>
+      <c r="W63" s="161"/>
+      <c r="X63" s="161"/>
+      <c r="Y63" s="161"/>
+      <c r="Z63" s="161"/>
+      <c r="AA63" s="161"/>
+      <c r="AB63" s="161"/>
+      <c r="AC63" s="161"/>
+      <c r="AD63" s="161"/>
+      <c r="AE63" s="161"/>
+      <c r="AF63" s="161"/>
+      <c r="AG63" s="161"/>
+      <c r="AH63" s="161"/>
+      <c r="AI63" s="161"/>
     </row>
     <row r="64" spans="1:35" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="160"/>
-      <c r="B64" s="160"/>
-      <c r="C64" s="160"/>
-      <c r="D64" s="160"/>
-      <c r="E64" s="160"/>
-      <c r="F64" s="160"/>
-      <c r="G64" s="160"/>
-      <c r="H64" s="160"/>
-      <c r="I64" s="160"/>
-      <c r="J64" s="160"/>
-      <c r="K64" s="160"/>
-      <c r="L64" s="160"/>
-      <c r="M64" s="160"/>
-      <c r="N64" s="160"/>
-      <c r="O64" s="160"/>
-      <c r="P64" s="160"/>
-      <c r="Q64" s="160"/>
-      <c r="R64" s="160"/>
-      <c r="S64" s="160"/>
-      <c r="T64" s="160"/>
-      <c r="U64" s="160"/>
-      <c r="V64" s="160"/>
-      <c r="W64" s="160"/>
-      <c r="X64" s="160"/>
-      <c r="Y64" s="160"/>
-      <c r="Z64" s="160"/>
-      <c r="AA64" s="160"/>
-      <c r="AB64" s="160"/>
-      <c r="AC64" s="160"/>
-      <c r="AD64" s="160"/>
-      <c r="AE64" s="160"/>
-      <c r="AF64" s="160"/>
-      <c r="AG64" s="160"/>
-      <c r="AH64" s="160"/>
-      <c r="AI64" s="160"/>
+      <c r="A64" s="162"/>
+      <c r="B64" s="162"/>
+      <c r="C64" s="162"/>
+      <c r="D64" s="162"/>
+      <c r="E64" s="162"/>
+      <c r="F64" s="162"/>
+      <c r="G64" s="162"/>
+      <c r="H64" s="162"/>
+      <c r="I64" s="162"/>
+      <c r="J64" s="162"/>
+      <c r="K64" s="162"/>
+      <c r="L64" s="162"/>
+      <c r="M64" s="162"/>
+      <c r="N64" s="162"/>
+      <c r="O64" s="162"/>
+      <c r="P64" s="162"/>
+      <c r="Q64" s="162"/>
+      <c r="R64" s="162"/>
+      <c r="S64" s="162"/>
+      <c r="T64" s="162"/>
+      <c r="U64" s="162"/>
+      <c r="V64" s="162"/>
+      <c r="W64" s="162"/>
+      <c r="X64" s="162"/>
+      <c r="Y64" s="162"/>
+      <c r="Z64" s="162"/>
+      <c r="AA64" s="162"/>
+      <c r="AB64" s="162"/>
+      <c r="AC64" s="162"/>
+      <c r="AD64" s="162"/>
+      <c r="AE64" s="162"/>
+      <c r="AF64" s="162"/>
+      <c r="AG64" s="162"/>
+      <c r="AH64" s="162"/>
+      <c r="AI64" s="162"/>
     </row>
     <row r="65" spans="1:37" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="157" t="s">
+      <c r="A65" s="159" t="s">
         <v>39</v>
       </c>
-      <c r="B65" s="157"/>
-      <c r="C65" s="157"/>
-      <c r="D65" s="157"/>
-      <c r="E65" s="157"/>
-      <c r="F65" s="157"/>
-      <c r="G65" s="157"/>
-      <c r="H65" s="157"/>
-      <c r="I65" s="157"/>
-      <c r="J65" s="157"/>
-      <c r="K65" s="157"/>
-      <c r="L65" s="157"/>
-      <c r="M65" s="157"/>
-      <c r="N65" s="157"/>
-      <c r="O65" s="157"/>
-      <c r="P65" s="157"/>
-      <c r="Q65" s="157"/>
-      <c r="R65" s="157"/>
-      <c r="S65" s="157"/>
-      <c r="T65" s="157"/>
-      <c r="U65" s="157"/>
-      <c r="V65" s="157"/>
-      <c r="W65" s="157"/>
-      <c r="X65" s="157"/>
-      <c r="Y65" s="157"/>
-      <c r="Z65" s="157"/>
-      <c r="AA65" s="157"/>
-      <c r="AB65" s="157"/>
-      <c r="AC65" s="157"/>
-      <c r="AD65" s="157"/>
-      <c r="AE65" s="157"/>
-      <c r="AF65" s="157"/>
-      <c r="AG65" s="157"/>
-      <c r="AH65" s="157"/>
-      <c r="AI65" s="157"/>
+      <c r="B65" s="159"/>
+      <c r="C65" s="159"/>
+      <c r="D65" s="159"/>
+      <c r="E65" s="159"/>
+      <c r="F65" s="159"/>
+      <c r="G65" s="159"/>
+      <c r="H65" s="159"/>
+      <c r="I65" s="159"/>
+      <c r="J65" s="159"/>
+      <c r="K65" s="159"/>
+      <c r="L65" s="159"/>
+      <c r="M65" s="159"/>
+      <c r="N65" s="159"/>
+      <c r="O65" s="159"/>
+      <c r="P65" s="159"/>
+      <c r="Q65" s="159"/>
+      <c r="R65" s="159"/>
+      <c r="S65" s="159"/>
+      <c r="T65" s="159"/>
+      <c r="U65" s="159"/>
+      <c r="V65" s="159"/>
+      <c r="W65" s="159"/>
+      <c r="X65" s="159"/>
+      <c r="Y65" s="159"/>
+      <c r="Z65" s="159"/>
+      <c r="AA65" s="159"/>
+      <c r="AB65" s="159"/>
+      <c r="AC65" s="159"/>
+      <c r="AD65" s="159"/>
+      <c r="AE65" s="159"/>
+      <c r="AF65" s="159"/>
+      <c r="AG65" s="159"/>
+      <c r="AH65" s="159"/>
+      <c r="AI65" s="159"/>
     </row>
     <row r="66" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A66" s="156" t="s">
+      <c r="A66" s="158" t="s">
         <v>56</v>
       </c>
-      <c r="B66" s="156"/>
-      <c r="C66" s="156"/>
-      <c r="D66" s="156"/>
-      <c r="E66" s="156"/>
-      <c r="F66" s="156"/>
-      <c r="G66" s="156"/>
-      <c r="H66" s="156"/>
-      <c r="I66" s="156"/>
-      <c r="J66" s="156"/>
-      <c r="K66" s="156"/>
-      <c r="L66" s="156"/>
-      <c r="M66" s="156"/>
-      <c r="N66" s="156"/>
-      <c r="O66" s="156"/>
-      <c r="P66" s="156"/>
-      <c r="Q66" s="156"/>
-      <c r="R66" s="156"/>
-      <c r="S66" s="156"/>
-      <c r="T66" s="156"/>
-      <c r="U66" s="156"/>
-      <c r="V66" s="156"/>
-      <c r="W66" s="156"/>
-      <c r="X66" s="156"/>
-      <c r="Y66" s="156"/>
-      <c r="Z66" s="156"/>
-      <c r="AA66" s="156"/>
-      <c r="AB66" s="156"/>
-      <c r="AC66" s="156"/>
-      <c r="AD66" s="156"/>
-      <c r="AE66" s="156"/>
-      <c r="AF66" s="156"/>
-      <c r="AG66" s="156"/>
-      <c r="AH66" s="156"/>
-      <c r="AI66" s="156"/>
+      <c r="B66" s="158"/>
+      <c r="C66" s="158"/>
+      <c r="D66" s="158"/>
+      <c r="E66" s="158"/>
+      <c r="F66" s="158"/>
+      <c r="G66" s="158"/>
+      <c r="H66" s="158"/>
+      <c r="I66" s="158"/>
+      <c r="J66" s="158"/>
+      <c r="K66" s="158"/>
+      <c r="L66" s="158"/>
+      <c r="M66" s="158"/>
+      <c r="N66" s="158"/>
+      <c r="O66" s="158"/>
+      <c r="P66" s="158"/>
+      <c r="Q66" s="158"/>
+      <c r="R66" s="158"/>
+      <c r="S66" s="158"/>
+      <c r="T66" s="158"/>
+      <c r="U66" s="158"/>
+      <c r="V66" s="158"/>
+      <c r="W66" s="158"/>
+      <c r="X66" s="158"/>
+      <c r="Y66" s="158"/>
+      <c r="Z66" s="158"/>
+      <c r="AA66" s="158"/>
+      <c r="AB66" s="158"/>
+      <c r="AC66" s="158"/>
+      <c r="AD66" s="158"/>
+      <c r="AE66" s="158"/>
+      <c r="AF66" s="158"/>
+      <c r="AG66" s="158"/>
+      <c r="AH66" s="158"/>
+      <c r="AI66" s="158"/>
       <c r="AJ66" s="84"/>
     </row>
     <row r="72" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="C72" s="137"/>
-      <c r="D72" s="137"/>
-      <c r="E72" s="137"/>
-      <c r="F72" s="137"/>
-      <c r="G72" s="137"/>
-      <c r="H72" s="137"/>
-      <c r="I72" s="137"/>
-      <c r="J72" s="137"/>
-      <c r="K72" s="137"/>
-      <c r="L72" s="137"/>
-      <c r="M72" s="137"/>
-      <c r="N72" s="137"/>
-      <c r="O72" s="137"/>
-      <c r="P72" s="137"/>
-      <c r="Q72" s="137"/>
-      <c r="R72" s="137"/>
-      <c r="S72" s="137"/>
-      <c r="T72" s="137"/>
-      <c r="U72" s="137"/>
-      <c r="V72" s="137"/>
-      <c r="W72" s="137"/>
-      <c r="X72" s="137"/>
-      <c r="Y72" s="137"/>
-      <c r="Z72" s="137"/>
-      <c r="AA72" s="137"/>
-      <c r="AB72" s="137"/>
-      <c r="AC72" s="137"/>
-      <c r="AD72" s="137"/>
-      <c r="AE72" s="137"/>
-      <c r="AF72" s="137"/>
-      <c r="AG72" s="137"/>
-      <c r="AH72" s="137"/>
-      <c r="AI72" s="137"/>
-      <c r="AJ72" s="137"/>
-      <c r="AK72" s="137"/>
+      <c r="C72" s="138"/>
+      <c r="D72" s="138"/>
+      <c r="E72" s="138"/>
+      <c r="F72" s="138"/>
+      <c r="G72" s="138"/>
+      <c r="H72" s="138"/>
+      <c r="I72" s="138"/>
+      <c r="J72" s="138"/>
+      <c r="K72" s="138"/>
+      <c r="L72" s="138"/>
+      <c r="M72" s="138"/>
+      <c r="N72" s="138"/>
+      <c r="O72" s="138"/>
+      <c r="P72" s="138"/>
+      <c r="Q72" s="138"/>
+      <c r="R72" s="138"/>
+      <c r="S72" s="138"/>
+      <c r="T72" s="138"/>
+      <c r="U72" s="138"/>
+      <c r="V72" s="138"/>
+      <c r="W72" s="138"/>
+      <c r="X72" s="138"/>
+      <c r="Y72" s="138"/>
+      <c r="Z72" s="138"/>
+      <c r="AA72" s="138"/>
+      <c r="AB72" s="138"/>
+      <c r="AC72" s="138"/>
+      <c r="AD72" s="138"/>
+      <c r="AE72" s="138"/>
+      <c r="AF72" s="138"/>
+      <c r="AG72" s="138"/>
+      <c r="AH72" s="138"/>
+      <c r="AI72" s="138"/>
+      <c r="AJ72" s="138"/>
+      <c r="AK72" s="138"/>
     </row>
     <row r="73" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="C73" s="137"/>
-      <c r="D73" s="137"/>
-      <c r="E73" s="137"/>
-      <c r="F73" s="137"/>
-      <c r="G73" s="137"/>
-      <c r="H73" s="137"/>
-      <c r="I73" s="137"/>
-      <c r="J73" s="137"/>
-      <c r="K73" s="137"/>
-      <c r="L73" s="137"/>
-      <c r="M73" s="137"/>
-      <c r="N73" s="137"/>
-      <c r="O73" s="137"/>
-      <c r="P73" s="137"/>
-      <c r="Q73" s="137"/>
-      <c r="R73" s="137"/>
-      <c r="S73" s="137"/>
-      <c r="T73" s="137"/>
-      <c r="U73" s="137"/>
-      <c r="V73" s="137"/>
-      <c r="W73" s="137"/>
-      <c r="X73" s="137"/>
-      <c r="Y73" s="137"/>
-      <c r="Z73" s="137"/>
-      <c r="AA73" s="137"/>
-      <c r="AB73" s="137"/>
-      <c r="AC73" s="137"/>
-      <c r="AD73" s="137"/>
-      <c r="AE73" s="137"/>
-      <c r="AF73" s="137"/>
-      <c r="AG73" s="137"/>
-      <c r="AH73" s="137"/>
-      <c r="AI73" s="137"/>
-      <c r="AJ73" s="137"/>
-      <c r="AK73" s="137"/>
+      <c r="C73" s="138"/>
+      <c r="D73" s="138"/>
+      <c r="E73" s="138"/>
+      <c r="F73" s="138"/>
+      <c r="G73" s="138"/>
+      <c r="H73" s="138"/>
+      <c r="I73" s="138"/>
+      <c r="J73" s="138"/>
+      <c r="K73" s="138"/>
+      <c r="L73" s="138"/>
+      <c r="M73" s="138"/>
+      <c r="N73" s="138"/>
+      <c r="O73" s="138"/>
+      <c r="P73" s="138"/>
+      <c r="Q73" s="138"/>
+      <c r="R73" s="138"/>
+      <c r="S73" s="138"/>
+      <c r="T73" s="138"/>
+      <c r="U73" s="138"/>
+      <c r="V73" s="138"/>
+      <c r="W73" s="138"/>
+      <c r="X73" s="138"/>
+      <c r="Y73" s="138"/>
+      <c r="Z73" s="138"/>
+      <c r="AA73" s="138"/>
+      <c r="AB73" s="138"/>
+      <c r="AC73" s="138"/>
+      <c r="AD73" s="138"/>
+      <c r="AE73" s="138"/>
+      <c r="AF73" s="138"/>
+      <c r="AG73" s="138"/>
+      <c r="AH73" s="138"/>
+      <c r="AI73" s="138"/>
+      <c r="AJ73" s="138"/>
+      <c r="AK73" s="138"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="RuEKvU7/dJ0hwmz5mxXRgZtzgNynla/w7eQBTe0PcGWTXxklaT60oRsfO0v95pgnReb5WHV5zlnthxZ1XkzvUQ==" saltValue="WfE36dWj1bQNM3GI3XWOPQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
-  <protectedRanges>
-    <protectedRange sqref="V57 A60:A62 N60:T62 U57:U62 W57:AI62 V59:V62 C72:AK73 A44 L44:AJ45 A65:AI65 B45:B47 C44:E45 G44:H45 AD46:AJ47 C46:D47" name="Диапазон7"/>
-    <protectedRange sqref="B57 B42:D43 E42:F42 J42 F43:S43 A52:A62 B58:C58 D57:D58 E57:F57 J57 F58:T58 AI53:AI56 Z52:AI52 M52:X52" name="Диапазон6"/>
-    <protectedRange sqref="A48:P48 Y48:AI48 Y49:Y51 Z51 A49:A50 A51:B51 P49:P51 Q48:X51" name="Диапазон5"/>
-    <protectedRange sqref="A1" name="Диапазон2"/>
-    <protectedRange sqref="A1 A39:E40 F40 AI39 A41:H41 AG11:AG13 AG39 K12:V12 P15:AI15 A14:N15 A11:I13 U16:AI17 A42:A43 A45:A47 AI29:AI31 A27:L28 N27:Q28 S27:S28 AI18:AI20 N16:Q17 S16:S17 A16:L17 A18:B20 A29:B31 U27:AI28" name="Диапазон1"/>
-    <protectedRange sqref="C20 G20 K20 O20 S20 W20 AA20 AE20 C31 G31 K31 S31 W31 AA31 AE31 O31" name="Диапазон4_1"/>
-    <protectedRange sqref="B53:B54 R55:U55 C56:Q56 X56:Y56 W55:AB55 AD55:AH56 D53:Q54" name="Диапазон2_4"/>
-    <protectedRange sqref="X53:X54 R53:V54" name="Диапазон5_4"/>
-    <protectedRange sqref="A63:AI64" name="Диапазон7_3"/>
-    <protectedRange sqref="E46:I47 J47 L46 V46:W46 N47:W47" name="Диапазон7_2_2_2"/>
-    <protectedRange sqref="X47:AC47" name="Диапазон2_4_2_1_2"/>
-    <protectedRange sqref="Y46" name="Диапазон5_4_2_1_2"/>
-  </protectedRanges>
-  <mergeCells count="187">
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="Q7:R7"/>
-    <mergeCell ref="A1:AI1"/>
-    <mergeCell ref="A2:AI3"/>
-    <mergeCell ref="B5:I5"/>
-    <mergeCell ref="J5:V5"/>
-    <mergeCell ref="W5:X5"/>
-    <mergeCell ref="J6:V6"/>
-    <mergeCell ref="K12:V12"/>
-    <mergeCell ref="AD9:AE9"/>
-    <mergeCell ref="AG9:AH9"/>
-    <mergeCell ref="B11:J11"/>
-    <mergeCell ref="K11:V11"/>
-    <mergeCell ref="W11:X11"/>
-    <mergeCell ref="B9:H9"/>
-    <mergeCell ref="I9:M9"/>
-    <mergeCell ref="O9:Y9"/>
-    <mergeCell ref="AA9:AB9"/>
-    <mergeCell ref="AD10:AE10"/>
-    <mergeCell ref="B14:L14"/>
-    <mergeCell ref="M14:AH14"/>
-    <mergeCell ref="I10:M10"/>
-    <mergeCell ref="O10:Y10"/>
-    <mergeCell ref="AA10:AB10"/>
-    <mergeCell ref="AG10:AH10"/>
-    <mergeCell ref="C19:J19"/>
-    <mergeCell ref="K19:R19"/>
-    <mergeCell ref="S19:Z19"/>
-    <mergeCell ref="AA19:AH19"/>
-    <mergeCell ref="M15:AH15"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="F16:J16"/>
-    <mergeCell ref="K16:P16"/>
-    <mergeCell ref="Q16:R16"/>
-    <mergeCell ref="S16:T16"/>
-    <mergeCell ref="U16:Y16"/>
-    <mergeCell ref="Z16:AA16"/>
-    <mergeCell ref="AB16:AF16"/>
-    <mergeCell ref="AG16:AH16"/>
-    <mergeCell ref="AE20:AF20"/>
-    <mergeCell ref="AG20:AH20"/>
-    <mergeCell ref="S20:T20"/>
-    <mergeCell ref="U20:V20"/>
-    <mergeCell ref="W20:X20"/>
-    <mergeCell ref="Y20:Z20"/>
-    <mergeCell ref="AC22:AD22"/>
-    <mergeCell ref="AF22:AH22"/>
-    <mergeCell ref="B17:AH17"/>
-    <mergeCell ref="C18:J18"/>
-    <mergeCell ref="K18:R18"/>
-    <mergeCell ref="S18:Z18"/>
-    <mergeCell ref="AA18:AH18"/>
-    <mergeCell ref="AA20:AB20"/>
-    <mergeCell ref="AC20:AD20"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="O20:P20"/>
-    <mergeCell ref="Q20:R20"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="I20:J20"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="Ppi9nK1tD2xs3OeijpWp3iPpeni3wNacfsIxzIjA8k9y7/+l/nq9nPWq1GtBGJrJTh9hWDk+58lfbyDV1JJXEA==" saltValue="SnvKn/a+ogY06ewWkYJxEg==" spinCount="100000" sheet="1" objects="1" scenarios="1" formatCells="0"/>
+  <mergeCells count="188">
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="O31:P31"/>
+    <mergeCell ref="AA31:AB31"/>
+    <mergeCell ref="B33:K33"/>
+    <mergeCell ref="M33:U33"/>
+    <mergeCell ref="W33:X33"/>
+    <mergeCell ref="M35:U35"/>
+    <mergeCell ref="W35:X35"/>
+    <mergeCell ref="Z35:AA35"/>
+    <mergeCell ref="AC35:AD35"/>
+    <mergeCell ref="AF35:AH35"/>
+    <mergeCell ref="AF34:AH34"/>
+    <mergeCell ref="B37:AH37"/>
+    <mergeCell ref="B39:I39"/>
+    <mergeCell ref="G43:I43"/>
+    <mergeCell ref="K43:S43"/>
+    <mergeCell ref="J40:V40"/>
+    <mergeCell ref="B41:AA41"/>
+    <mergeCell ref="W42:AH42"/>
+    <mergeCell ref="AF36:AH36"/>
+    <mergeCell ref="J39:V39"/>
+    <mergeCell ref="W39:X39"/>
+    <mergeCell ref="W34:X34"/>
+    <mergeCell ref="Z34:AA34"/>
+    <mergeCell ref="AC34:AD34"/>
+    <mergeCell ref="W40:X40"/>
+    <mergeCell ref="Q52:X52"/>
+    <mergeCell ref="X46:Y46"/>
+    <mergeCell ref="X47:Y47"/>
+    <mergeCell ref="Z47:AA47"/>
+    <mergeCell ref="AB47:AC47"/>
+    <mergeCell ref="B35:K35"/>
+    <mergeCell ref="B49:O50"/>
+    <mergeCell ref="Q49:X51"/>
+    <mergeCell ref="Z49:AH50"/>
+    <mergeCell ref="B51:O51"/>
+    <mergeCell ref="W43:AH43"/>
+    <mergeCell ref="W36:X36"/>
+    <mergeCell ref="Z36:AA36"/>
+    <mergeCell ref="AC36:AD36"/>
+    <mergeCell ref="J47:W47"/>
+    <mergeCell ref="A44:D45"/>
+    <mergeCell ref="E44:AI44"/>
+    <mergeCell ref="E45:AI45"/>
+    <mergeCell ref="E46:L46"/>
+    <mergeCell ref="M46:U46"/>
+    <mergeCell ref="V46:W46"/>
+    <mergeCell ref="Z46:AA46"/>
+    <mergeCell ref="AB46:AC46"/>
+    <mergeCell ref="Z51:AH51"/>
+    <mergeCell ref="C72:AK73"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="V57:AI60"/>
+    <mergeCell ref="G58:I58"/>
+    <mergeCell ref="K58:S58"/>
+    <mergeCell ref="B59:M59"/>
+    <mergeCell ref="B60:M60"/>
+    <mergeCell ref="AD53:AH53"/>
+    <mergeCell ref="R55:U56"/>
+    <mergeCell ref="W55:X55"/>
+    <mergeCell ref="Y55:Z55"/>
+    <mergeCell ref="AA55:AB55"/>
+    <mergeCell ref="AD55:AH56"/>
+    <mergeCell ref="R53:U53"/>
+    <mergeCell ref="W53:X53"/>
+    <mergeCell ref="Y53:Z53"/>
+    <mergeCell ref="AA53:AB53"/>
+    <mergeCell ref="A66:AI66"/>
+    <mergeCell ref="A65:AI65"/>
+    <mergeCell ref="B56:P56"/>
+    <mergeCell ref="A63:AI64"/>
+    <mergeCell ref="B55:O55"/>
+    <mergeCell ref="B61:M61"/>
+    <mergeCell ref="B62:M62"/>
+    <mergeCell ref="AC33:AD33"/>
+    <mergeCell ref="AF33:AH33"/>
+    <mergeCell ref="Q27:R27"/>
+    <mergeCell ref="S27:T27"/>
+    <mergeCell ref="Q31:R31"/>
+    <mergeCell ref="S31:T31"/>
+    <mergeCell ref="K29:R29"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="K30:R30"/>
+    <mergeCell ref="S30:Z30"/>
+    <mergeCell ref="AA30:AH30"/>
+    <mergeCell ref="K27:P27"/>
+    <mergeCell ref="Z27:AA27"/>
+    <mergeCell ref="AB27:AF27"/>
+    <mergeCell ref="AG27:AH27"/>
+    <mergeCell ref="B28:AH28"/>
+    <mergeCell ref="U27:Y27"/>
+    <mergeCell ref="AA29:AH29"/>
+    <mergeCell ref="S29:Z29"/>
+    <mergeCell ref="C30:J30"/>
+    <mergeCell ref="Z33:AA33"/>
+    <mergeCell ref="U31:V31"/>
+    <mergeCell ref="W31:X31"/>
+    <mergeCell ref="Y31:Z31"/>
     <mergeCell ref="AC24:AD24"/>
     <mergeCell ref="AF24:AH24"/>
     <mergeCell ref="AC31:AD31"/>
@@ -5541,138 +5626,96 @@
     <mergeCell ref="Z25:AA25"/>
     <mergeCell ref="C29:J29"/>
     <mergeCell ref="W25:X25"/>
-    <mergeCell ref="AC33:AD33"/>
-    <mergeCell ref="AF33:AH33"/>
-    <mergeCell ref="Q27:R27"/>
-    <mergeCell ref="S27:T27"/>
-    <mergeCell ref="Q31:R31"/>
-    <mergeCell ref="S31:T31"/>
-    <mergeCell ref="K29:R29"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="K30:R30"/>
-    <mergeCell ref="S30:Z30"/>
-    <mergeCell ref="AA30:AH30"/>
-    <mergeCell ref="K27:P27"/>
-    <mergeCell ref="Z27:AA27"/>
-    <mergeCell ref="AB27:AF27"/>
-    <mergeCell ref="AG27:AH27"/>
-    <mergeCell ref="B28:AH28"/>
-    <mergeCell ref="U27:Y27"/>
-    <mergeCell ref="AA29:AH29"/>
-    <mergeCell ref="S29:Z29"/>
-    <mergeCell ref="C30:J30"/>
-    <mergeCell ref="Z33:AA33"/>
-    <mergeCell ref="U31:V31"/>
-    <mergeCell ref="W31:X31"/>
-    <mergeCell ref="Y31:Z31"/>
-    <mergeCell ref="C72:AK73"/>
-    <mergeCell ref="B57:D57"/>
-    <mergeCell ref="V57:AI60"/>
-    <mergeCell ref="G58:I58"/>
-    <mergeCell ref="K58:S58"/>
-    <mergeCell ref="B59:M59"/>
-    <mergeCell ref="B60:M60"/>
-    <mergeCell ref="AD53:AH53"/>
-    <mergeCell ref="R55:U56"/>
-    <mergeCell ref="W55:X55"/>
-    <mergeCell ref="Y55:Z55"/>
-    <mergeCell ref="AA55:AB55"/>
-    <mergeCell ref="AD55:AH56"/>
-    <mergeCell ref="R53:U53"/>
-    <mergeCell ref="W53:X53"/>
-    <mergeCell ref="Y53:Z53"/>
-    <mergeCell ref="AA53:AB53"/>
-    <mergeCell ref="A66:AI66"/>
-    <mergeCell ref="A65:AI65"/>
-    <mergeCell ref="B56:P56"/>
-    <mergeCell ref="A63:AI64"/>
-    <mergeCell ref="B55:O55"/>
-    <mergeCell ref="B61:M61"/>
-    <mergeCell ref="B62:M62"/>
-    <mergeCell ref="Q52:X52"/>
-    <mergeCell ref="X46:Y46"/>
-    <mergeCell ref="X47:Y47"/>
-    <mergeCell ref="Z47:AA47"/>
-    <mergeCell ref="AB47:AC47"/>
-    <mergeCell ref="B35:K35"/>
-    <mergeCell ref="B49:O50"/>
-    <mergeCell ref="Q49:X51"/>
-    <mergeCell ref="Z49:AH50"/>
-    <mergeCell ref="B51:O51"/>
-    <mergeCell ref="W43:AH43"/>
-    <mergeCell ref="W36:X36"/>
-    <mergeCell ref="Z36:AA36"/>
-    <mergeCell ref="AC36:AD36"/>
-    <mergeCell ref="J47:W47"/>
-    <mergeCell ref="A44:D45"/>
-    <mergeCell ref="E44:AI44"/>
-    <mergeCell ref="E45:AI45"/>
-    <mergeCell ref="E46:L46"/>
-    <mergeCell ref="M46:U46"/>
-    <mergeCell ref="V46:W46"/>
-    <mergeCell ref="Z46:AA46"/>
-    <mergeCell ref="AB46:AC46"/>
-    <mergeCell ref="Z51:AH51"/>
-    <mergeCell ref="M35:U35"/>
-    <mergeCell ref="W35:X35"/>
-    <mergeCell ref="Z35:AA35"/>
-    <mergeCell ref="AC35:AD35"/>
-    <mergeCell ref="AF35:AH35"/>
-    <mergeCell ref="AF34:AH34"/>
-    <mergeCell ref="B37:AH37"/>
-    <mergeCell ref="B39:I39"/>
-    <mergeCell ref="G43:I43"/>
-    <mergeCell ref="K43:S43"/>
-    <mergeCell ref="J40:V40"/>
-    <mergeCell ref="B41:AA41"/>
-    <mergeCell ref="W42:AH42"/>
-    <mergeCell ref="AF36:AH36"/>
-    <mergeCell ref="J39:V39"/>
-    <mergeCell ref="W39:X39"/>
-    <mergeCell ref="W34:X34"/>
-    <mergeCell ref="Z34:AA34"/>
-    <mergeCell ref="AC34:AD34"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="O31:P31"/>
-    <mergeCell ref="AA31:AB31"/>
-    <mergeCell ref="B33:K33"/>
-    <mergeCell ref="M33:U33"/>
-    <mergeCell ref="W33:X33"/>
+    <mergeCell ref="AE20:AF20"/>
+    <mergeCell ref="AG20:AH20"/>
+    <mergeCell ref="S20:T20"/>
+    <mergeCell ref="U20:V20"/>
+    <mergeCell ref="W20:X20"/>
+    <mergeCell ref="Y20:Z20"/>
+    <mergeCell ref="AC22:AD22"/>
+    <mergeCell ref="AF22:AH22"/>
+    <mergeCell ref="B17:AH17"/>
+    <mergeCell ref="C18:J18"/>
+    <mergeCell ref="K18:R18"/>
+    <mergeCell ref="S18:Z18"/>
+    <mergeCell ref="AA18:AH18"/>
+    <mergeCell ref="AA20:AB20"/>
+    <mergeCell ref="AC20:AD20"/>
+    <mergeCell ref="K20:L20"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="O20:P20"/>
+    <mergeCell ref="Q20:R20"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="B14:L14"/>
+    <mergeCell ref="M14:AH14"/>
+    <mergeCell ref="I10:M10"/>
+    <mergeCell ref="O10:Y10"/>
+    <mergeCell ref="AA10:AB10"/>
+    <mergeCell ref="AG10:AH10"/>
+    <mergeCell ref="C19:J19"/>
+    <mergeCell ref="K19:R19"/>
+    <mergeCell ref="S19:Z19"/>
+    <mergeCell ref="AA19:AH19"/>
+    <mergeCell ref="M15:AH15"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="F16:J16"/>
+    <mergeCell ref="K16:P16"/>
+    <mergeCell ref="Q16:R16"/>
+    <mergeCell ref="S16:T16"/>
+    <mergeCell ref="U16:Y16"/>
+    <mergeCell ref="Z16:AA16"/>
+    <mergeCell ref="AB16:AF16"/>
+    <mergeCell ref="AG16:AH16"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="Q7:R7"/>
+    <mergeCell ref="A1:AI1"/>
+    <mergeCell ref="A2:AI3"/>
+    <mergeCell ref="B5:I5"/>
+    <mergeCell ref="J5:V5"/>
+    <mergeCell ref="W5:X5"/>
+    <mergeCell ref="J6:V6"/>
+    <mergeCell ref="K12:V12"/>
+    <mergeCell ref="AD9:AE9"/>
+    <mergeCell ref="AG9:AH9"/>
+    <mergeCell ref="B11:J11"/>
+    <mergeCell ref="K11:V11"/>
+    <mergeCell ref="W11:X11"/>
+    <mergeCell ref="B9:H9"/>
+    <mergeCell ref="I9:M9"/>
+    <mergeCell ref="O9:Y9"/>
+    <mergeCell ref="AA9:AB9"/>
+    <mergeCell ref="AD10:AE10"/>
   </mergeCells>
-  <dataValidations count="10">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R53:U54">
+  <dataValidations count="9">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R53:U54" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>$AN$6:$AN$8</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA54:AB54">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA54:AB54" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>$AR$6:$AR$34</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y53:Z54 Z46:AA46">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y53:Z54 Z46:AA46" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>$AQ$6:$AQ$17</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W53:X54 X46:Y46">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W53:X54 X46:Y46" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>$AP$6:$AP$36</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M14:AH14">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M14:AH14" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>$AK$6:$AK$8</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Z16:AA16 Z27:AA27">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Z16:AA16 Z27:AA27" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>$AL$6:$AL$11</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AG16:AH16 AG27:AH27">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AG16:AH16 AG27:AH27" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>$AM$6:$AM$15</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y5:AH5 D7:P7 S7:AA7 Y11:AH11 Y39:AH39 G42:I42 K42:M42 O42:P42 R42:S42 G57:I57 K57:M57 O57:P57 R57:S57">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y5:AH5 D7:P7 S7:AA7 Y11:AH11 Y39:AH40 G42:I42 K42:M42 O42:P42 R42:S42 G57:I57 K57:M57 O57:P57 R57:S57" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>0</formula1>
       <formula2>9</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA53:AB53">
-      <formula1>$AR$6:$AR$37</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AB46:AC46">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA53:AB53 AB46:AC46" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>$AR$6:$AR$37</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>